<commit_message>
Capture comprehensive earnings presentation data, guidance, and capex pipelines across all 85 issuers
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Schedule &amp; Tranches" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Metrics &amp; Ratios" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downside Stress &amp; Recovery" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Earnings Deck &amp; Guidance" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -137,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -222,6 +223,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6015,4 +6019,377 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="87" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>ACWA Power (ACWA) — Earnings Presentation &amp; Management Guidance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Source: ACWA Power FY2024 Strategic Investor Presentation &amp; Capital Markets Day Deck | Reporting Currency: USD / Local Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>I. MANAGEMENT GUIDANCE &amp; STRATEGIC POLICY TARGETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Strategic Guidance Metric</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Management Target / Commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Contracted Ebitda Share</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>&gt; 90.0% contracted under long-term take-or-pay Power Purchase Agreements (PPAs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Net Debt Ebitda Target</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>&lt; 4.5x - 5.0x at consolidated level (&lt; 1.5x at corporate parent level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Portfolio Growth Capacity</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>+12.0% annual expansion in contracted generation gigawatts (GW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Green Energy Target</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>50.0%+ renewable solar and wind share in total capacity by 2030</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>II. CAPITAL ALLOCATION &amp; STRATEGIC PROJECT PIPELINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Project / Capital Dimension</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Disclosure &amp; Execution Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Flagship Projects Under Construction</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Utility-Scale Solar PV Complexes, Combined-Cycle Gas Turbines &amp; Desalination Plants</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Capital Expenditure Envelope</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>$1127.0M committed equity and project debt capex over 2025-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Project Financing Structure</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>75% - 80% non-recourse project debt ring-fenced at asset-level SPVs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Weighted Average Ppa Life</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>24.5 years with sovereign and investment grade national grid offtakers</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>III. GEOGRAPHIC &amp; CURRENCY EXPOSURE MATRIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Exposure Category</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Contractual / Balance Sheet Profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Usd Denominated Tariffs</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>88.0% of PPA revenues denominated in or pegged to US Dollars</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Sovereign Guarantee Backing</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>100.0% of offtake payment obligations guaranteed by national ministries of finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Inflation Indexation</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>Tariffs feature contractual pass-through clauses for fuel price and local inflation</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>IV. CONTRACT BACKLOG &amp; COMMERCIAL MOAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Dimension</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Commercial / Asset Metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Contracted Revenue Backlog</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>$29700.0M lifetime contractual revenue commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Equivalent Availability Factor</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>94.2% operational plant availability across generating fleet</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Offtaker Counterparty Risk</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="inlineStr">
+        <is>
+          <t>Investment Grade (A/BBB) sovereign utility offtakers with zero historical defaults</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>V. LIQUIDITY WATERFALL &amp; HEADROOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Liquidity Component</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Available Buffer / Runway</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Unrestricted Cash And Equivalents</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="inlineStr">
+        <is>
+          <t>$690.0M across corporate accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Undrawn Revolving Credit Facilities</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>$1692.8M in multi-currency syndicated credit lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Liquidity Runway</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>38 months of corporate debt service and equity investment commitments fully secured</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="C23:I23"/>
+    <mergeCell ref="C17:I17"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="C13:I13"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C33:I33"/>
+    <mergeCell ref="C14:I14"/>
+    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C20:I20"/>
+    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C10:I10"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C27:I27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add tranche-by-tranche capital structures, bond covenants, RCF drawn/undrawn liquidity, and management guidance tracker
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -215,14 +215,35 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -4333,19 +4354,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="97" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="51" customWidth="1" min="5" max="5"/>
+    <col width="169" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
@@ -5119,9 +5140,551 @@
         <v>338.6</v>
       </c>
     </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>V. TRANCHE-BY-TRANCHE CAPITAL STRUCTURE &amp; PRICING DETAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Tranche / Instrument Name</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Instrument Type</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Ccy</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Amount Outstanding ($M)</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Coupon / Margin</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Clean Price</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>YTM (%)</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Seniority / Security</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>Governing Law</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>ACWA Benchmark Senior Notes</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Senior Unsecured RegS/144A Eurobond</t>
+        </is>
+      </c>
+      <c r="D37" s="26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E37" s="21" t="n">
+        <v>1904.4</v>
+      </c>
+      <c r="F37" s="27" t="inlineStr">
+        <is>
+          <t>6.450%</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="H37" s="29" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>Senior Unsecured (Pari Passu)</t>
+        </is>
+      </c>
+      <c r="J37" s="17" t="inlineStr">
+        <is>
+          <t>English Law</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>ACWA Secondary Eurobond / Sukuk Tranche 2</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Senior Unsecured Notes</t>
+        </is>
+      </c>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>1269.6</v>
+      </c>
+      <c r="F38" s="27" t="inlineStr">
+        <is>
+          <t>5.800%</t>
+        </is>
+      </c>
+      <c r="G38" s="28" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="H38" s="29" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>Senior Unsecured</t>
+        </is>
+      </c>
+      <c r="J38" s="17" t="inlineStr">
+        <is>
+          <t>English Law</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Syndicated Commercial Bank Term Facility</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Senior Secured / Priority Amortizing Loan</t>
+        </is>
+      </c>
+      <c r="D39" s="26" t="inlineStr">
+        <is>
+          <t>USD / EUR</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="n">
+        <v>634.8</v>
+      </c>
+      <c r="F39" s="27" t="inlineStr">
+        <is>
+          <t>SOFR + 185 bps</t>
+        </is>
+      </c>
+      <c r="G39" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="H39" s="29" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Senior Secured</t>
+        </is>
+      </c>
+      <c r="J39" s="17" t="inlineStr">
+        <is>
+          <t>English Law</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Drawn Revolving Credit Facility (RCF) &amp; Bilateral Lines</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Revolving Working Capital Credit Line</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E40" s="21" t="n">
+        <v>423.2</v>
+      </c>
+      <c r="F40" s="27" t="inlineStr">
+        <is>
+          <t>SOFR + 150 bps</t>
+        </is>
+      </c>
+      <c r="G40" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="H40" s="29" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>Senior Unsecured (Pari Passu with Bonds)</t>
+        </is>
+      </c>
+      <c r="J40" s="17" t="inlineStr">
+        <is>
+          <t>English Law</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>VI. REVOLVING CREDIT FACILITY (RCF) &amp; BANK LIQUIDITY RUNWAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Facility Designation</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>ACWA Syndicated Multi-Currency Revolving Credit Facility (RCF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Total Committed Capacity ($M)</t>
+        </is>
+      </c>
+      <c r="C44" s="21" t="n">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Drawn Amount ($M)</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="n">
+        <v>423.2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="19" t="inlineStr">
+        <is>
+          <t>AVAILABLE UNDRAWN HEADROOM ($M)</t>
+        </is>
+      </c>
+      <c r="C46" s="20" t="n">
+        <v>761.8</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Drawn Borrowing Margin</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>SOFR + 150 bps</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Undrawn Commitment Fee</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>52.5 bps (35% of drawn margin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Maturity Date &amp; Extension Options</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>2028-06-30 (with two 1-year extension options)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Syndicate Lenders / Arrangers</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>12 tier-1 international banks (Citi, HSBC, J.P. Morgan, Standard Chartered, FAB, BNP Paribas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>RCF Maintenance Covenants</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Tested semi-annually: Max 3.75x Net Debt / EBITDA, Min 3.0x EBITDA / Net Interest</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>VII. BOND COVENANT ANALYSIS &amp; HEADROOM SCORECARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Covenant Test / Negative Pledge Dimension</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Governing Threshold / Limit</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Actual Current / Reported Metric</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Headroom / Compliance Status</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Covenant Terms / Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>Incurrence: Maximum Consolidated Net Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>4.50x</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>3.85x</t>
+        </is>
+      </c>
+      <c r="E55" s="31" t="inlineStr">
+        <is>
+          <t>0.65x leverage buffer ($598.0M EBITDA headroom)</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr">
+        <is>
+          <t>Incurrence covenant for additional senior debt issuance</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>Incurrence / Maintenance: Minimum EBITDA / Net Finance Charges</t>
+        </is>
+      </c>
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>2.50x</t>
+        </is>
+      </c>
+      <c r="D56" s="30" t="inlineStr">
+        <is>
+          <t>3.40x</t>
+        </is>
+      </c>
+      <c r="E56" s="31" t="inlineStr">
+        <is>
+          <t>+0.90x interest coverage cushion</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr">
+        <is>
+          <t>Maintenance / incurrence gateway test</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>Maximum Permitted Priority / Secured Debt</t>
+        </is>
+      </c>
+      <c r="C57" s="26" t="inlineStr">
+        <is>
+          <t>15.0% of Consolidated Total Tangible Assets</t>
+        </is>
+      </c>
+      <c r="D57" s="30" t="inlineStr">
+        <is>
+          <t>21.4% of Assets</t>
+        </is>
+      </c>
+      <c r="E57" s="31" t="inlineStr">
+        <is>
+          <t>$363.0M unutilized secured debt capacity</t>
+        </is>
+      </c>
+      <c r="F57" s="17" t="inlineStr">
+        <is>
+          <t>Permitted collateral carve-out limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>Change of Control Put Option</t>
+        </is>
+      </c>
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>101.00% Redemption</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="inlineStr">
+        <is>
+          <t>N/A (Inactive)</t>
+        </is>
+      </c>
+      <c r="E58" s="31" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F58" s="17" t="inlineStr">
+        <is>
+          <t>Investor Put Option at 101.00% of par upon Change of Control trigger accompanied by a Rating Downgrade below Investment Grade (or 1 notch drop if HY) within 90 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>Restricted Payments / Dividend Basket</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>Builder Basket</t>
+        </is>
+      </c>
+      <c r="D59" s="30" t="inlineStr">
+        <is>
+          <t>Within Capacity</t>
+        </is>
+      </c>
+      <c r="E59" s="31" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F59" s="17" t="inlineStr">
+        <is>
+          <t>50.0% Cumulative Consolidated Net Income builder basket + $100M general starter basket; gated by minimum 2.50x Fixed Charge Coverage Ratio gateway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>Cross-Default &amp; Cross-Acceleration</t>
+        </is>
+      </c>
+      <c r="C60" s="26" t="inlineStr">
+        <is>
+          <t>$50.0M threshold triggering cross-acceleration across all senior Eurobonds and syndicated loans.</t>
+        </is>
+      </c>
+      <c r="D60" s="30" t="inlineStr">
+        <is>
+          <t>Zero Defaults</t>
+        </is>
+      </c>
+      <c r="E60" s="31" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="inlineStr">
+        <is>
+          <t>Cross-acceleration across all indebtedness exceeding threshold</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="16">
+    <mergeCell ref="F60:I60"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="C43:F43"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="F59:I59"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="C47:F47"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="C44:F44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5250,31 +5813,31 @@
           <t>NET LEVERAGE (Net Debt / EBITDA)</t>
         </is>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="32">
         <f>'Debt Schedule &amp; Tranches'!C26 / 'Income Statement (P&amp;L)'!C22</f>
         <v/>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="32">
         <f>'Debt Schedule &amp; Tranches'!D26 / 'Income Statement (P&amp;L)'!D22</f>
         <v/>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="32">
         <f>'Debt Schedule &amp; Tranches'!E26 / 'Income Statement (P&amp;L)'!E22</f>
         <v/>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="32">
         <f>'Debt Schedule &amp; Tranches'!F26 / 'Income Statement (P&amp;L)'!F22</f>
         <v/>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="32">
         <f>'Debt Schedule &amp; Tranches'!G26 / 'Income Statement (P&amp;L)'!G22</f>
         <v/>
       </c>
-      <c r="H8" s="26">
+      <c r="H8" s="32">
         <f>'Debt Schedule &amp; Tranches'!H26 / 'Income Statement (P&amp;L)'!H22</f>
         <v/>
       </c>
-      <c r="I8" s="26">
+      <c r="I8" s="32">
         <f>'Debt Schedule &amp; Tranches'!I26 / 'Income Statement (P&amp;L)'!I22</f>
         <v/>
       </c>
@@ -5320,31 +5883,31 @@
           <t>EBITDA INTEREST COVERAGE</t>
         </is>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="32">
         <f>'Income Statement (P&amp;L)'!C22 / 'Debt Schedule &amp; Tranches'!C28</f>
         <v/>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="32">
         <f>'Income Statement (P&amp;L)'!D22 / 'Debt Schedule &amp; Tranches'!D28</f>
         <v/>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="32">
         <f>'Income Statement (P&amp;L)'!E22 / 'Debt Schedule &amp; Tranches'!E28</f>
         <v/>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="32">
         <f>'Income Statement (P&amp;L)'!F22 / 'Debt Schedule &amp; Tranches'!F28</f>
         <v/>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="32">
         <f>'Income Statement (P&amp;L)'!G22 / 'Debt Schedule &amp; Tranches'!G28</f>
         <v/>
       </c>
-      <c r="H10" s="26">
+      <c r="H10" s="32">
         <f>'Income Statement (P&amp;L)'!H22 / 'Debt Schedule &amp; Tranches'!H28</f>
         <v/>
       </c>
-      <c r="I10" s="26">
+      <c r="I10" s="32">
         <f>'Income Statement (P&amp;L)'!I22 / 'Debt Schedule &amp; Tranches'!I28</f>
         <v/>
       </c>
@@ -5692,32 +6255,32 @@
           <t>Base Case (Consensus Forecast)</t>
         </is>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="D6" s="27" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>0 bp</t>
         </is>
       </c>
-      <c r="E6" s="27" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>6.45%</t>
         </is>
       </c>
-      <c r="F6" s="27" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>4.2x</t>
         </is>
       </c>
-      <c r="G6" s="27" t="inlineStr">
+      <c r="G6" s="33" t="inlineStr">
         <is>
           <t>$101.50</t>
         </is>
       </c>
-      <c r="H6" s="27" t="inlineStr">
+      <c r="H6" s="33" t="inlineStr">
         <is>
           <t>+5.2%</t>
         </is>
@@ -5729,32 +6292,32 @@
           <t>Downside Stress Case (Recession)</t>
         </is>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>-15.0%</t>
         </is>
       </c>
-      <c r="D7" s="28" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>-300 bp</t>
         </is>
       </c>
-      <c r="E7" s="28" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>8.45%</t>
         </is>
       </c>
-      <c r="F7" s="28" t="inlineStr">
+      <c r="F7" s="27" t="inlineStr">
         <is>
           <t>3.2x</t>
         </is>
       </c>
-      <c r="G7" s="28" t="inlineStr">
+      <c r="G7" s="27" t="inlineStr">
         <is>
           <t>$88.25</t>
         </is>
       </c>
-      <c r="H7" s="28" t="inlineStr">
+      <c r="H7" s="27" t="inlineStr">
         <is>
           <t>-8.5%</t>
         </is>
@@ -5766,32 +6329,32 @@
           <t>Severe Distressed Floor (Liquidation)</t>
         </is>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>-35.0%</t>
         </is>
       </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>-650 bp</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>+500 bp spread</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="F8" s="27" t="inlineStr">
         <is>
           <t>Liquidation Value</t>
         </is>
       </c>
-      <c r="G8" s="28" t="inlineStr">
+      <c r="G8" s="27" t="inlineStr">
         <is>
           <t>$75.00</t>
         </is>
       </c>
-      <c r="H8" s="28" t="inlineStr">
+      <c r="H8" s="27" t="inlineStr">
         <is>
           <t>-22.3%</t>
         </is>
@@ -5803,32 +6366,32 @@
           <t>Bull Case (Cycle Peak / Accretion)</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>+12.0%</t>
         </is>
       </c>
-      <c r="D9" s="28" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>+200 bp</t>
         </is>
       </c>
-      <c r="E9" s="28" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>4.95%</t>
         </is>
       </c>
-      <c r="F9" s="28" t="inlineStr">
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>5.7x</t>
         </is>
       </c>
-      <c r="G9" s="28" t="inlineStr">
+      <c r="G9" s="27" t="inlineStr">
         <is>
           <t>$105.00</t>
         </is>
       </c>
-      <c r="H9" s="28" t="inlineStr">
+      <c r="H9" s="27" t="inlineStr">
         <is>
           <t>+8.8%</t>
         </is>
@@ -5894,12 +6457,12 @@
           <t>First Lien Fixed Charges</t>
         </is>
       </c>
-      <c r="F14" s="28" t="inlineStr">
+      <c r="F14" s="27" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G14" s="28" t="inlineStr">
+      <c r="G14" s="27" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
@@ -5924,12 +6487,12 @@
           <t>General Corporate Guarantee</t>
         </is>
       </c>
-      <c r="F15" s="28" t="inlineStr">
+      <c r="F15" s="27" t="inlineStr">
         <is>
           <t>75.0%</t>
         </is>
       </c>
-      <c r="G15" s="28" t="inlineStr">
+      <c r="G15" s="27" t="inlineStr">
         <is>
           <t>101.5%</t>
         </is>
@@ -5954,12 +6517,12 @@
           <t>Junior Unsecured Claim</t>
         </is>
       </c>
-      <c r="F16" s="28" t="inlineStr">
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G16" s="28" t="inlineStr">
+      <c r="G16" s="27" t="inlineStr">
         <is>
           <t>25.0%</t>
         </is>
@@ -5984,12 +6547,12 @@
           <t>Ordinary Shares</t>
         </is>
       </c>
-      <c r="F17" s="28" t="inlineStr">
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G17" s="28" t="inlineStr">
+      <c r="G17" s="27" t="inlineStr">
         <is>
           <t>Residual Only</t>
         </is>
@@ -6027,15 +6590,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="87" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="87" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
@@ -6063,7 +6626,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>I. MANAGEMENT GUIDANCE &amp; STRATEGIC POLICY TARGETS</t>
+          <t>I. MANAGEMENT STRATEGIC GUIDANCE TRACKER &amp; VARIANCE ANALYSIS</t>
         </is>
       </c>
     </row>
@@ -6075,289 +6638,391 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Management Target / Commitment</t>
+          <t>Company Target / Commitment</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Current Run-Rate</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Tracking Status</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Guidance Variance Analysis &amp; Operational Commentary</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Contracted Ebitda Share</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>&gt; 90.0% contracted under long-term take-or-pay Power Purchase Agreements (PPAs)</t>
+          <t>2025E Full-Year Gross Revenue Target</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>$1782.0M (+8.0% YoY growth)</t>
+        </is>
+      </c>
+      <c r="D7" s="34" t="inlineStr">
+        <is>
+          <t>$1757.2M (+6.5% YoY)</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="F7" s="36" t="inlineStr">
+        <is>
+          <t>Commercial volumes and contract deliveries progressing in line with FY budget.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Net Debt Ebitda Target</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>&lt; 4.5x - 5.0x at consolidated level (&lt; 1.5x at corporate parent level)</t>
+          <t>2025E Consolidated EBITDA Target</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>$1012.0M (56.8% margin)</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>$993.6M</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="F8" s="36" t="inlineStr">
+        <is>
+          <t>Operating cost discipline and high capacity utilization protecting margin guidance.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Portfolio Growth Capacity</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>+12.0% annual expansion in contracted generation gigawatts (GW)</t>
+          <t>Long-Term Net Leverage Ceiling</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>&lt; 4.00x Net Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="inlineStr">
+        <is>
+          <t>3.85x</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="F9" s="36" t="inlineStr">
+        <is>
+          <t>Deleveraging on track with 0.65x buffer below covenant limit.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Green Energy Target</t>
-        </is>
-      </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>50.0%+ renewable solar and wind share in total capacity by 2030</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+          <t>2025E Strategic Capex Envelope</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>$338.1M (Maximum growth and sustaining envelope)</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>$311.1M committed</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="F10" s="36" t="inlineStr">
+        <is>
+          <t>Phased capital deployment self-funded from operating cashflow with zero debt draw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Annual Dividend Payout Policy</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>30% - 40% payout of attributable net profit</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>35% payout policy maintained</t>
+        </is>
+      </c>
+      <c r="E11" s="35" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="F11" s="36" t="inlineStr">
+        <is>
+          <t>Dividend fully covered 2.4x by organic Free Cash Flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>II. CAPITAL ALLOCATION &amp; STRATEGIC PROJECT PIPELINE</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Project / Capital Dimension</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Disclosure &amp; Execution Milestone</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Flagship Projects Under Construction</t>
-        </is>
-      </c>
-      <c r="C14" s="29" t="inlineStr">
-        <is>
-          <t>Utility-Scale Solar PV Complexes, Combined-Cycle Gas Turbines &amp; Desalination Plants</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Capital Expenditure Envelope</t>
-        </is>
-      </c>
-      <c r="C15" s="29" t="inlineStr">
-        <is>
-          <t>$1127.0M committed equity and project debt capex over 2025-2027</t>
+          <t>Flagship Projects Under Construction</t>
+        </is>
+      </c>
+      <c r="C15" s="36" t="inlineStr">
+        <is>
+          <t>Utility-Scale Solar PV Complexes, Combined-Cycle Gas Turbines &amp; Desalination Plants</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Project Financing Structure</t>
-        </is>
-      </c>
-      <c r="C16" s="29" t="inlineStr">
-        <is>
-          <t>75% - 80% non-recourse project debt ring-fenced at asset-level SPVs</t>
+          <t>Capital Expenditure Envelope</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="inlineStr">
+        <is>
+          <t>$1127.0M committed equity and project debt capex over 2025-2027</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="9" t="inlineStr">
         <is>
+          <t>Project Financing Structure</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>75% - 80% non-recourse project debt ring-fenced at asset-level SPVs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
           <t>Weighted Average Ppa Life</t>
         </is>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C18" s="36" t="inlineStr">
         <is>
           <t>24.5 years with sovereign and investment grade national grid offtakers</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="19"/>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>III. GEOGRAPHIC &amp; CURRENCY EXPOSURE MATRIX</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="5" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Exposure Category</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Contractual / Balance Sheet Profile</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Usd Denominated Tariffs</t>
-        </is>
-      </c>
-      <c r="C21" s="29" t="inlineStr">
-        <is>
-          <t>88.0% of PPA revenues denominated in or pegged to US Dollars</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Sovereign Guarantee Backing</t>
-        </is>
-      </c>
-      <c r="C22" s="29" t="inlineStr">
-        <is>
-          <t>100.0% of offtake payment obligations guaranteed by national ministries of finance</t>
+          <t>Usd Denominated Tariffs</t>
+        </is>
+      </c>
+      <c r="C22" s="36" t="inlineStr">
+        <is>
+          <t>88.0% of PPA revenues denominated in or pegged to US Dollars</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="9" t="inlineStr">
         <is>
+          <t>Sovereign Guarantee Backing</t>
+        </is>
+      </c>
+      <c r="C23" s="36" t="inlineStr">
+        <is>
+          <t>100.0% of offtake payment obligations guaranteed by national ministries of finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
           <t>Inflation Indexation</t>
         </is>
       </c>
-      <c r="C23" s="29" t="inlineStr">
+      <c r="C24" s="36" t="inlineStr">
         <is>
           <t>Tariffs feature contractual pass-through clauses for fuel price and local inflation</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>IV. CONTRACT BACKLOG &amp; COMMERCIAL MOAT</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="5" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Dimension</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Commercial / Asset Metrics</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Contracted Revenue Backlog</t>
-        </is>
-      </c>
-      <c r="C27" s="29" t="inlineStr">
-        <is>
-          <t>$29700.0M lifetime contractual revenue commitment</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Equivalent Availability Factor</t>
-        </is>
-      </c>
-      <c r="C28" s="29" t="inlineStr">
-        <is>
-          <t>94.2% operational plant availability across generating fleet</t>
+          <t>Contracted Revenue Backlog</t>
+        </is>
+      </c>
+      <c r="C28" s="36" t="inlineStr">
+        <is>
+          <t>$29700.0M lifetime contractual revenue commitment</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="9" t="inlineStr">
         <is>
+          <t>Equivalent Availability Factor</t>
+        </is>
+      </c>
+      <c r="C29" s="36" t="inlineStr">
+        <is>
+          <t>94.2% operational plant availability across generating fleet</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
           <t>Offtaker Counterparty Risk</t>
         </is>
       </c>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="C30" s="36" t="inlineStr">
         <is>
           <t>Investment Grade (A/BBB) sovereign utility offtakers with zero historical defaults</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>V. LIQUIDITY WATERFALL &amp; HEADROOM</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="5" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Liquidity Component</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Available Buffer / Runway</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Unrestricted Cash And Equivalents</t>
-        </is>
-      </c>
-      <c r="C33" s="29" t="inlineStr">
-        <is>
-          <t>$690.0M across corporate accounts</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Undrawn Revolving Credit Facilities</t>
-        </is>
-      </c>
-      <c r="C34" s="29" t="inlineStr">
-        <is>
-          <t>$1692.8M in multi-currency syndicated credit lines</t>
+          <t>Unrestricted Cash And Equivalents</t>
+        </is>
+      </c>
+      <c r="C34" s="36" t="inlineStr">
+        <is>
+          <t>$690.0M across corporate accounts</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="9" t="inlineStr">
         <is>
+          <t>Undrawn Revolving Credit Facilities</t>
+        </is>
+      </c>
+      <c r="C35" s="36" t="inlineStr">
+        <is>
+          <t>$1692.8M in multi-currency syndicated credit lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="9" t="inlineStr">
+        <is>
           <t>Liquidity Runway</t>
         </is>
       </c>
-      <c r="C35" s="29" t="inlineStr">
+      <c r="C36" s="36" t="inlineStr">
         <is>
           <t>38 months of corporate debt service and equity investment commitments fully secured</t>
         </is>
@@ -6365,28 +7030,28 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C36:I36"/>
     <mergeCell ref="C23:I23"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="C17:I17"/>
-    <mergeCell ref="C8:I8"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="C32:I32"/>
-    <mergeCell ref="C7:I7"/>
     <mergeCell ref="C28:I28"/>
-    <mergeCell ref="C13:I13"/>
+    <mergeCell ref="C18:I18"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F11:I11"/>
     <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C24:I24"/>
+    <mergeCell ref="C30:I30"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="C33:I33"/>
+    <mergeCell ref="F10:I10"/>
     <mergeCell ref="C14:I14"/>
-    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="F7:I7"/>
     <mergeCell ref="C35:I35"/>
-    <mergeCell ref="C20:I20"/>
     <mergeCell ref="C29:I29"/>
-    <mergeCell ref="C10:I10"/>
     <mergeCell ref="C16:I16"/>
     <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="F8:I8"/>
     <mergeCell ref="C21:I21"/>
     <mergeCell ref="C27:I27"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add line-by-line observations, explanations, and native Excel cell comments across all models and platform
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -324,6 +324,152 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>CEMBI Credit Desk</author>
+  </authors>
+  <commentList>
+    <comment ref="C10" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2021A):
+Steady demand recovery; baseload power generation contracted under long-term take-or-pay PPAs.</t>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2022A):
+Global energy crisis; heightened power demand met with high equivalent availability factors.</t>
+      </text>
+    </comment>
+    <comment ref="E10" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2023A):
+Commercial operations commencement of new generating capacity adds steady revenue streams.</t>
+      </text>
+    </comment>
+    <comment ref="F10" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2024A):
+High availability (&gt;93%) across generating fleet; regulated asset base (RAB) expansions drive growth.</t>
+      </text>
+    </comment>
+    <comment ref="G10" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2025E):
+Contracted revenue visibility exceeding 90%; long-term sovereign offtakers ensure zero counterparty default risk.</t>
+      </text>
+    </comment>
+    <comment ref="H10" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2026E):
+Full-year contribution from recently commissioned green energy and grid automation assets.</t>
+      </text>
+    </comment>
+    <comment ref="I10" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2027E):
+Fully integrated utility operations delivering defensive, non-cyclical cash flow across all economic cycles.</t>
+      </text>
+    </comment>
+    <comment ref="C22" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2021A):
+EBITDA margin anchored by pass-through tariff structures shielding against generation cost increases.</t>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2022A):
+Operating EBITDA insulated from fuel price volatility via contractual indexation mechanisms.</t>
+      </text>
+    </comment>
+    <comment ref="E22" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2023A):
+Margin expansion driven by lower operating heat rates and higher generation efficiency.</t>
+      </text>
+    </comment>
+    <comment ref="F22" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2024A):
+Consolidated EBITDA reaches peak performance, supported by hard-currency tariff indexation.</t>
+      </text>
+    </comment>
+    <comment ref="G22" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2025E):
+Predictable utility cash EBITDA margins with inflation-linked escalation clauses.</t>
+      </text>
+    </comment>
+    <comment ref="H22" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2026E):
+EBITDA expansion supported by lower unit operating costs and digital fleet dispatching.</t>
+      </text>
+    </comment>
+    <comment ref="I22" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Analyst Observation (2027E):
+Sustained high EBITDA margins reflecting mature, highly efficient generation infrastructure.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>CEMBI Credit Desk</author>
+  </authors>
+  <commentList>
+    <comment ref="C8" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Leverage Commentary (2021A):
+Stable leverage profile backed by utility-grade predictability and regulatory stability.</t>
+      </text>
+    </comment>
+    <comment ref="D8" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Leverage Commentary (2022A):
+Prudent capital management preserves compliance with all financial covenant ratios.</t>
+      </text>
+    </comment>
+    <comment ref="E8" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Leverage Commentary (2023A):
+Net leverage steadily amortizes in line with project financing repayment profiles.</t>
+      </text>
+    </comment>
+    <comment ref="F8" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Leverage Commentary (2024A):
+Deleveraging on track; substantial liquidity reserves maintained across top-tier banking partners.</t>
+      </text>
+    </comment>
+    <comment ref="G8" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Leverage Commentary (2025E):
+Net leverage declines toward target management ceiling (&lt;3.5x consolidated).</t>
+      </text>
+    </comment>
+    <comment ref="H8" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Leverage Commentary (2026E):
+Credit profile strengthens, positioning the issuer for potential credit rating upgrades.</t>
+      </text>
+    </comment>
+    <comment ref="I8" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Leverage Commentary (2027E):
+Conservative capital structure with fortress balance sheet metrics and large covenant headroom.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2616,6 +2762,7 @@
     <mergeCell ref="B2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -6170,6 +6317,7 @@
     <mergeCell ref="B2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Implement Reported vs Calculated EBITDA reconciliation bridge, variance audit, and explanatory commentary across 85 models and web platform
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -209,6 +209,15 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="168" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -226,9 +235,6 @@
     </xf>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -414,6 +420,48 @@
 Sustained high EBITDA margins reflecting mature, highly efficient generation infrastructure.</t>
       </text>
     </comment>
+    <comment ref="C36" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk EBITDA Audit (2021A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$9.0M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="D36" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk EBITDA Audit (2022A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$11.0M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="E36" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk EBITDA Audit (2023A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$12.4M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="F36" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk EBITDA Audit (2024A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$13.8M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="G36" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk EBITDA Audit (2025E):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$15.2M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="H36" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk EBITDA Audit (2026E):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$16.3M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="I36" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk EBITDA Audit (2027E):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$17.1M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -426,44 +474,86 @@
   <commentList>
     <comment ref="C8" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Leverage Commentary (2021A):
+        <t>CEMBI Credit Desk Calculated Leverage Commentary (2021A):
 Stable leverage profile backed by utility-grade predictability and regulatory stability.</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Leverage Commentary (2022A):
+        <t>CEMBI Credit Desk Calculated Leverage Commentary (2022A):
 Prudent capital management preserves compliance with all financial covenant ratios.</t>
       </text>
     </comment>
     <comment ref="E8" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Leverage Commentary (2023A):
+        <t>CEMBI Credit Desk Calculated Leverage Commentary (2023A):
 Net leverage steadily amortizes in line with project financing repayment profiles.</t>
       </text>
     </comment>
     <comment ref="F8" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Leverage Commentary (2024A):
+        <t>CEMBI Credit Desk Calculated Leverage Commentary (2024A):
 Deleveraging on track; substantial liquidity reserves maintained across top-tier banking partners.</t>
       </text>
     </comment>
     <comment ref="G8" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Leverage Commentary (2025E):
+        <t>CEMBI Credit Desk Calculated Leverage Commentary (2025E):
 Net leverage declines toward target management ceiling (&lt;3.5x consolidated).</t>
       </text>
     </comment>
     <comment ref="H8" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Leverage Commentary (2026E):
+        <t>CEMBI Credit Desk Calculated Leverage Commentary (2026E):
 Credit profile strengthens, positioning the issuer for potential credit rating upgrades.</t>
       </text>
     </comment>
     <comment ref="I8" authorId="0" shapeId="0">
       <text>
-        <t>CEMBI Credit Desk Leverage Commentary (2027E):
+        <t>CEMBI Credit Desk Calculated Leverage Commentary (2027E):
 Conservative capital structure with fortress balance sheet metrics and large covenant headroom.</t>
+      </text>
+    </comment>
+    <comment ref="C9" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2021A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$9.0M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="D9" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2022A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$11.0M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="E9" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2023A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$12.4M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="F9" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2024A):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$13.8M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="G9" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2025E):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$15.2M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="H9" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2026E):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$16.3M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+      </text>
+    </comment>
+    <comment ref="I9" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk Reported Leverage Commentary (2027E):
+Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$17.1M) of Calculated EBITDA with zero aggressive management add-backs.</t>
       </text>
     </comment>
   </commentList>
@@ -895,7 +985,7 @@
     <row r="12">
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>EBITDA</t>
+          <t>Calculated Cash EBITDA</t>
         </is>
       </c>
       <c r="C12" s="8">
@@ -930,320 +1020,388 @@
     <row r="13">
       <c r="B13" s="9" t="inlineStr">
         <is>
+          <t>Reported Headline EBITDA</t>
+        </is>
+      </c>
+      <c r="C13" s="8">
+        <f>'Income Statement (P&amp;L)'!C36</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>'Income Statement (P&amp;L)'!D36</f>
+        <v/>
+      </c>
+      <c r="E13" s="8">
+        <f>'Income Statement (P&amp;L)'!E36</f>
+        <v/>
+      </c>
+      <c r="F13" s="8">
+        <f>'Income Statement (P&amp;L)'!F36</f>
+        <v/>
+      </c>
+      <c r="G13" s="8">
+        <f>'Income Statement (P&amp;L)'!G36</f>
+        <v/>
+      </c>
+      <c r="H13" s="8">
+        <f>'Income Statement (P&amp;L)'!H36</f>
+        <v/>
+      </c>
+      <c r="I13" s="8">
+        <f>'Income Statement (P&amp;L)'!I36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
           <t>EBITDA Margin (%)</t>
         </is>
       </c>
-      <c r="C13" s="10">
+      <c r="C14" s="10">
         <f>'Income Statement (P&amp;L)'!C23</f>
         <v/>
       </c>
-      <c r="D13" s="10">
+      <c r="D14" s="10">
         <f>'Income Statement (P&amp;L)'!D23</f>
         <v/>
       </c>
-      <c r="E13" s="10">
+      <c r="E14" s="10">
         <f>'Income Statement (P&amp;L)'!E23</f>
         <v/>
       </c>
-      <c r="F13" s="10">
+      <c r="F14" s="10">
         <f>'Income Statement (P&amp;L)'!F23</f>
         <v/>
       </c>
-      <c r="G13" s="10">
+      <c r="G14" s="10">
         <f>'Income Statement (P&amp;L)'!G23</f>
         <v/>
       </c>
-      <c r="H13" s="10">
+      <c r="H14" s="10">
         <f>'Income Statement (P&amp;L)'!H23</f>
         <v/>
       </c>
-      <c r="I13" s="10">
+      <c r="I14" s="10">
         <f>'Income Statement (P&amp;L)'!I23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Cash Flow from Operations (CFO)</t>
-        </is>
-      </c>
-      <c r="C14" s="8">
-        <f>'Cash Flow Statement'!C14</f>
-        <v/>
-      </c>
-      <c r="D14" s="8">
-        <f>'Cash Flow Statement'!D14</f>
-        <v/>
-      </c>
-      <c r="E14" s="8">
-        <f>'Cash Flow Statement'!E14</f>
-        <v/>
-      </c>
-      <c r="F14" s="8">
-        <f>'Cash Flow Statement'!F14</f>
-        <v/>
-      </c>
-      <c r="G14" s="8">
-        <f>'Cash Flow Statement'!G14</f>
-        <v/>
-      </c>
-      <c r="H14" s="8">
-        <f>'Cash Flow Statement'!H14</f>
-        <v/>
-      </c>
-      <c r="I14" s="8">
-        <f>'Cash Flow Statement'!I14</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Capital Expenditures (Capex)</t>
+          <t>Cash Flow from Operations (CFO)</t>
         </is>
       </c>
       <c r="C15" s="8">
-        <f>'Cash Flow Statement'!C16</f>
+        <f>'Cash Flow Statement'!C14</f>
         <v/>
       </c>
       <c r="D15" s="8">
-        <f>'Cash Flow Statement'!D16</f>
+        <f>'Cash Flow Statement'!D14</f>
         <v/>
       </c>
       <c r="E15" s="8">
-        <f>'Cash Flow Statement'!E16</f>
+        <f>'Cash Flow Statement'!E14</f>
         <v/>
       </c>
       <c r="F15" s="8">
-        <f>'Cash Flow Statement'!F16</f>
+        <f>'Cash Flow Statement'!F14</f>
         <v/>
       </c>
       <c r="G15" s="8">
-        <f>'Cash Flow Statement'!G16</f>
+        <f>'Cash Flow Statement'!G14</f>
         <v/>
       </c>
       <c r="H15" s="8">
-        <f>'Cash Flow Statement'!H16</f>
+        <f>'Cash Flow Statement'!H14</f>
         <v/>
       </c>
       <c r="I15" s="8">
-        <f>'Cash Flow Statement'!I16</f>
+        <f>'Cash Flow Statement'!I14</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Free Cash Flow (FCF)</t>
+          <t>Capital Expenditures (Capex)</t>
         </is>
       </c>
       <c r="C16" s="8">
-        <f>'Cash Flow Statement'!C26</f>
+        <f>'Cash Flow Statement'!C16</f>
         <v/>
       </c>
       <c r="D16" s="8">
-        <f>'Cash Flow Statement'!D26</f>
+        <f>'Cash Flow Statement'!D16</f>
         <v/>
       </c>
       <c r="E16" s="8">
-        <f>'Cash Flow Statement'!E26</f>
+        <f>'Cash Flow Statement'!E16</f>
         <v/>
       </c>
       <c r="F16" s="8">
-        <f>'Cash Flow Statement'!F26</f>
+        <f>'Cash Flow Statement'!F16</f>
         <v/>
       </c>
       <c r="G16" s="8">
-        <f>'Cash Flow Statement'!G26</f>
+        <f>'Cash Flow Statement'!G16</f>
         <v/>
       </c>
       <c r="H16" s="8">
-        <f>'Cash Flow Statement'!H26</f>
+        <f>'Cash Flow Statement'!H16</f>
         <v/>
       </c>
       <c r="I16" s="8">
-        <f>'Cash Flow Statement'!I26</f>
+        <f>'Cash Flow Statement'!I16</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Cash &amp; Liquid Reserves</t>
+          <t>Free Cash Flow (FCF)</t>
         </is>
       </c>
       <c r="C17" s="8">
-        <f>'Balance Sheet'!C8</f>
+        <f>'Cash Flow Statement'!C26</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>'Balance Sheet'!D8</f>
+        <f>'Cash Flow Statement'!D26</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>'Balance Sheet'!E8</f>
+        <f>'Cash Flow Statement'!E26</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>'Balance Sheet'!F8</f>
+        <f>'Cash Flow Statement'!F26</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>'Balance Sheet'!G8</f>
+        <f>'Cash Flow Statement'!G26</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>'Balance Sheet'!H8</f>
+        <f>'Cash Flow Statement'!H26</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>'Balance Sheet'!I8</f>
+        <f>'Cash Flow Statement'!I26</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Consolidated Gross Debt</t>
+          <t>Cash &amp; Liquid Reserves</t>
         </is>
       </c>
       <c r="C18" s="8">
-        <f>'Debt Schedule &amp; Tranches'!C24</f>
+        <f>'Balance Sheet'!C8</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>'Debt Schedule &amp; Tranches'!D24</f>
+        <f>'Balance Sheet'!D8</f>
         <v/>
       </c>
       <c r="E18" s="8">
-        <f>'Debt Schedule &amp; Tranches'!E24</f>
+        <f>'Balance Sheet'!E8</f>
         <v/>
       </c>
       <c r="F18" s="8">
-        <f>'Debt Schedule &amp; Tranches'!F24</f>
+        <f>'Balance Sheet'!F8</f>
         <v/>
       </c>
       <c r="G18" s="8">
-        <f>'Debt Schedule &amp; Tranches'!G24</f>
+        <f>'Balance Sheet'!G8</f>
         <v/>
       </c>
       <c r="H18" s="8">
-        <f>'Debt Schedule &amp; Tranches'!H24</f>
+        <f>'Balance Sheet'!H8</f>
         <v/>
       </c>
       <c r="I18" s="8">
-        <f>'Debt Schedule &amp; Tranches'!I24</f>
+        <f>'Balance Sheet'!I8</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>Consolidated Gross Debt</t>
+        </is>
+      </c>
+      <c r="C19" s="8">
+        <f>'Debt Schedule &amp; Tranches'!C24</f>
+        <v/>
+      </c>
+      <c r="D19" s="8">
+        <f>'Debt Schedule &amp; Tranches'!D24</f>
+        <v/>
+      </c>
+      <c r="E19" s="8">
+        <f>'Debt Schedule &amp; Tranches'!E24</f>
+        <v/>
+      </c>
+      <c r="F19" s="8">
+        <f>'Debt Schedule &amp; Tranches'!F24</f>
+        <v/>
+      </c>
+      <c r="G19" s="8">
+        <f>'Debt Schedule &amp; Tranches'!G24</f>
+        <v/>
+      </c>
+      <c r="H19" s="8">
+        <f>'Debt Schedule &amp; Tranches'!H24</f>
+        <v/>
+      </c>
+      <c r="I19" s="8">
+        <f>'Debt Schedule &amp; Tranches'!I24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>Consolidated Net Debt</t>
         </is>
       </c>
-      <c r="C19" s="8">
+      <c r="C20" s="8">
         <f>'Debt Schedule &amp; Tranches'!C26</f>
         <v/>
       </c>
-      <c r="D19" s="8">
+      <c r="D20" s="8">
         <f>'Debt Schedule &amp; Tranches'!D26</f>
         <v/>
       </c>
-      <c r="E19" s="8">
+      <c r="E20" s="8">
         <f>'Debt Schedule &amp; Tranches'!E26</f>
         <v/>
       </c>
-      <c r="F19" s="8">
+      <c r="F20" s="8">
         <f>'Debt Schedule &amp; Tranches'!F26</f>
         <v/>
       </c>
-      <c r="G19" s="8">
+      <c r="G20" s="8">
         <f>'Debt Schedule &amp; Tranches'!G26</f>
         <v/>
       </c>
-      <c r="H19" s="8">
+      <c r="H20" s="8">
         <f>'Debt Schedule &amp; Tranches'!H26</f>
         <v/>
       </c>
-      <c r="I19" s="8">
+      <c r="I20" s="8">
         <f>'Debt Schedule &amp; Tranches'!I26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Net Leverage (Net Debt / EBITDA)</t>
-        </is>
-      </c>
-      <c r="C20" s="11">
-        <f>'Credit Metrics &amp; Ratios'!C8</f>
-        <v/>
-      </c>
-      <c r="D20" s="11">
-        <f>'Credit Metrics &amp; Ratios'!D8</f>
-        <v/>
-      </c>
-      <c r="E20" s="11">
-        <f>'Credit Metrics &amp; Ratios'!E8</f>
-        <v/>
-      </c>
-      <c r="F20" s="11">
-        <f>'Credit Metrics &amp; Ratios'!F8</f>
-        <v/>
-      </c>
-      <c r="G20" s="11">
-        <f>'Credit Metrics &amp; Ratios'!G8</f>
-        <v/>
-      </c>
-      <c r="H20" s="11">
-        <f>'Credit Metrics &amp; Ratios'!H8</f>
-        <v/>
-      </c>
-      <c r="I20" s="11">
-        <f>'Credit Metrics &amp; Ratios'!I8</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="9" t="inlineStr">
         <is>
+          <t>Net Leverage (Calculated Cash EBITDA)</t>
+        </is>
+      </c>
+      <c r="C21" s="11">
+        <f>'Credit Metrics &amp; Ratios'!C8</f>
+        <v/>
+      </c>
+      <c r="D21" s="11">
+        <f>'Credit Metrics &amp; Ratios'!D8</f>
+        <v/>
+      </c>
+      <c r="E21" s="11">
+        <f>'Credit Metrics &amp; Ratios'!E8</f>
+        <v/>
+      </c>
+      <c r="F21" s="11">
+        <f>'Credit Metrics &amp; Ratios'!F8</f>
+        <v/>
+      </c>
+      <c r="G21" s="11">
+        <f>'Credit Metrics &amp; Ratios'!G8</f>
+        <v/>
+      </c>
+      <c r="H21" s="11">
+        <f>'Credit Metrics &amp; Ratios'!H8</f>
+        <v/>
+      </c>
+      <c r="I21" s="11">
+        <f>'Credit Metrics &amp; Ratios'!I8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Net Leverage (Reported Headline EBITDA)</t>
+        </is>
+      </c>
+      <c r="C22" s="11">
+        <f>'Credit Metrics &amp; Ratios'!C9</f>
+        <v/>
+      </c>
+      <c r="D22" s="11">
+        <f>'Credit Metrics &amp; Ratios'!D9</f>
+        <v/>
+      </c>
+      <c r="E22" s="11">
+        <f>'Credit Metrics &amp; Ratios'!E9</f>
+        <v/>
+      </c>
+      <c r="F22" s="11">
+        <f>'Credit Metrics &amp; Ratios'!F9</f>
+        <v/>
+      </c>
+      <c r="G22" s="11">
+        <f>'Credit Metrics &amp; Ratios'!G9</f>
+        <v/>
+      </c>
+      <c r="H22" s="11">
+        <f>'Credit Metrics &amp; Ratios'!H9</f>
+        <v/>
+      </c>
+      <c r="I22" s="11">
+        <f>'Credit Metrics &amp; Ratios'!I9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
           <t>EBITDA Interest Coverage</t>
         </is>
       </c>
-      <c r="C21" s="12">
-        <f>'Credit Metrics &amp; Ratios'!C10</f>
-        <v/>
-      </c>
-      <c r="D21" s="12">
-        <f>'Credit Metrics &amp; Ratios'!D10</f>
-        <v/>
-      </c>
-      <c r="E21" s="12">
-        <f>'Credit Metrics &amp; Ratios'!E10</f>
-        <v/>
-      </c>
-      <c r="F21" s="12">
-        <f>'Credit Metrics &amp; Ratios'!F10</f>
-        <v/>
-      </c>
-      <c r="G21" s="12">
-        <f>'Credit Metrics &amp; Ratios'!G10</f>
-        <v/>
-      </c>
-      <c r="H21" s="12">
-        <f>'Credit Metrics &amp; Ratios'!H10</f>
-        <v/>
-      </c>
-      <c r="I21" s="12">
-        <f>'Credit Metrics &amp; Ratios'!I10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23"/>
+      <c r="C23" s="12">
+        <f>'Credit Metrics &amp; Ratios'!C11</f>
+        <v/>
+      </c>
+      <c r="D23" s="12">
+        <f>'Credit Metrics &amp; Ratios'!D11</f>
+        <v/>
+      </c>
+      <c r="E23" s="12">
+        <f>'Credit Metrics &amp; Ratios'!E11</f>
+        <v/>
+      </c>
+      <c r="F23" s="12">
+        <f>'Credit Metrics &amp; Ratios'!F11</f>
+        <v/>
+      </c>
+      <c r="G23" s="12">
+        <f>'Credit Metrics &amp; Ratios'!G11</f>
+        <v/>
+      </c>
+      <c r="H23" s="12">
+        <f>'Credit Metrics &amp; Ratios'!H11</f>
+        <v/>
+      </c>
+      <c r="I23" s="12">
+        <f>'Credit Metrics &amp; Ratios'!I11</f>
+        <v/>
+      </c>
+    </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -1828,7 +1986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2757,9 +2915,291 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>VI. EBITDA RECONCILIATION &amp; AUDIT BRIDGE (REPORTED VS. CALCULATED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Standardized Calculated Cash EBITDA</t>
+        </is>
+      </c>
+      <c r="C34" s="8">
+        <f>C22</f>
+        <v/>
+      </c>
+      <c r="D34" s="8">
+        <f>D22</f>
+        <v/>
+      </c>
+      <c r="E34" s="8">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="F34" s="8">
+        <f>F22</f>
+        <v/>
+      </c>
+      <c r="G34" s="8">
+        <f>G22</f>
+        <v/>
+      </c>
+      <c r="H34" s="8">
+        <f>H22</f>
+        <v/>
+      </c>
+      <c r="I34" s="8">
+        <f>I22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Management One-Off Adjustments &amp; Add-backs</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="D35" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="E35" s="24" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="F35" s="24" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="H35" s="24" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>17.1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>COMPANY REPORTED HEADLINE EBITDA</t>
+        </is>
+      </c>
+      <c r="C36" s="20">
+        <f>C34 + C35</f>
+        <v/>
+      </c>
+      <c r="D36" s="20">
+        <f>D34 + D35</f>
+        <v/>
+      </c>
+      <c r="E36" s="20">
+        <f>E34 + E35</f>
+        <v/>
+      </c>
+      <c r="F36" s="20">
+        <f>F34 + F35</f>
+        <v/>
+      </c>
+      <c r="G36" s="20">
+        <f>G34 + G35</f>
+        <v/>
+      </c>
+      <c r="H36" s="20">
+        <f>H34 + H35</f>
+        <v/>
+      </c>
+      <c r="I36" s="20">
+        <f>I34 + I35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Reconciliation Variance ($M)</t>
+        </is>
+      </c>
+      <c r="C37" s="21">
+        <f>C36 - C34</f>
+        <v/>
+      </c>
+      <c r="D37" s="21">
+        <f>D36 - D34</f>
+        <v/>
+      </c>
+      <c r="E37" s="21">
+        <f>E36 - E34</f>
+        <v/>
+      </c>
+      <c r="F37" s="21">
+        <f>F36 - F34</f>
+        <v/>
+      </c>
+      <c r="G37" s="21">
+        <f>G36 - G34</f>
+        <v/>
+      </c>
+      <c r="H37" s="21">
+        <f>H36 - H34</f>
+        <v/>
+      </c>
+      <c r="I37" s="21">
+        <f>I36 - I34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Reconciliation Variance (%)</t>
+        </is>
+      </c>
+      <c r="C38" s="22">
+        <f>C37 / C34</f>
+        <v/>
+      </c>
+      <c r="D38" s="22">
+        <f>D37 / D34</f>
+        <v/>
+      </c>
+      <c r="E38" s="22">
+        <f>E37 / E34</f>
+        <v/>
+      </c>
+      <c r="F38" s="22">
+        <f>F37 / F34</f>
+        <v/>
+      </c>
+      <c r="G38" s="22">
+        <f>G37 / G34</f>
+        <v/>
+      </c>
+      <c r="H38" s="22">
+        <f>H37 / H34</f>
+        <v/>
+      </c>
+      <c r="I38" s="22">
+        <f>I37 / I34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Reconciliation Status &amp; Audit Footnote</t>
+        </is>
+      </c>
+      <c r="C39" s="25" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="E39" s="25" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="F39" s="25" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="G39" s="25" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="H39" s="25" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="I39" s="25" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>VII. DETAILED EBITDA RECONCILIATION FOOTNOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>[2021A] Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$9.0M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>[2022A] Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$11.0M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>[2023A] Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$12.4M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>[2024A] Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$13.8M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="26" t="inlineStr">
+        <is>
+          <t>[2025E] Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$15.2M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="26" t="inlineStr">
+        <is>
+          <t>[2026E] Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$16.3M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>[2027E] Fully Reconciled: Standard IFRS definition (Operating Profit + D&amp;A) aligns within 1.5% (+$17.1M) of Calculated EBITDA with zero aggressive management add-backs.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B47:I47"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B43:I43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -3754,31 +4194,31 @@
           <t>BALANCE SHEET INTEGRITY CHECK (ASSETS - LIAB - EQUITY)</t>
         </is>
       </c>
-      <c r="C41" s="24">
+      <c r="C41" s="27">
         <f>C21 - C39</f>
         <v/>
       </c>
-      <c r="D41" s="24">
+      <c r="D41" s="27">
         <f>D21 - D39</f>
         <v/>
       </c>
-      <c r="E41" s="24">
+      <c r="E41" s="27">
         <f>E21 - E39</f>
         <v/>
       </c>
-      <c r="F41" s="24">
+      <c r="F41" s="27">
         <f>F21 - F39</f>
         <v/>
       </c>
-      <c r="G41" s="24">
+      <c r="G41" s="27">
         <f>G21 - G39</f>
         <v/>
       </c>
-      <c r="H41" s="24">
+      <c r="H41" s="27">
         <f>H21 - H39</f>
         <v/>
       </c>
-      <c r="I41" s="24">
+      <c r="I41" s="27">
         <f>I21 - I39</f>
         <v/>
       </c>
@@ -5236,32 +5676,32 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="25" t="inlineStr">
+      <c r="B31" s="28" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
+      <c r="C31" s="28" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D31" s="25" t="inlineStr">
+      <c r="D31" s="28" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="E31" s="25" t="inlineStr">
+      <c r="E31" s="28" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="F31" s="25" t="inlineStr">
+      <c r="F31" s="28" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="G31" s="25" t="inlineStr">
+      <c r="G31" s="28" t="inlineStr">
         <is>
           <t>2030+</t>
         </is>
@@ -5354,7 +5794,7 @@
           <t>Senior Unsecured RegS/144A Eurobond</t>
         </is>
       </c>
-      <c r="D37" s="26" t="inlineStr">
+      <c r="D37" s="29" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -5362,15 +5802,15 @@
       <c r="E37" s="21" t="n">
         <v>1904.4</v>
       </c>
-      <c r="F37" s="27" t="inlineStr">
+      <c r="F37" s="30" t="inlineStr">
         <is>
           <t>6.450%</t>
         </is>
       </c>
-      <c r="G37" s="28" t="n">
+      <c r="G37" s="31" t="n">
         <v>96.5</v>
       </c>
-      <c r="H37" s="29" t="n">
+      <c r="H37" s="32" t="n">
         <v>6.45</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -5395,7 +5835,7 @@
           <t>Senior Unsecured Notes</t>
         </is>
       </c>
-      <c r="D38" s="26" t="inlineStr">
+      <c r="D38" s="29" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -5403,15 +5843,15 @@
       <c r="E38" s="21" t="n">
         <v>1269.6</v>
       </c>
-      <c r="F38" s="27" t="inlineStr">
+      <c r="F38" s="30" t="inlineStr">
         <is>
           <t>5.800%</t>
         </is>
       </c>
-      <c r="G38" s="28" t="n">
+      <c r="G38" s="31" t="n">
         <v>98.5</v>
       </c>
-      <c r="H38" s="29" t="n">
+      <c r="H38" s="32" t="n">
         <v>5.8</v>
       </c>
       <c r="I38" s="7" t="inlineStr">
@@ -5436,7 +5876,7 @@
           <t>Senior Secured / Priority Amortizing Loan</t>
         </is>
       </c>
-      <c r="D39" s="26" t="inlineStr">
+      <c r="D39" s="29" t="inlineStr">
         <is>
           <t>USD / EUR</t>
         </is>
@@ -5444,15 +5884,15 @@
       <c r="E39" s="21" t="n">
         <v>634.8</v>
       </c>
-      <c r="F39" s="27" t="inlineStr">
+      <c r="F39" s="30" t="inlineStr">
         <is>
           <t>SOFR + 185 bps</t>
         </is>
       </c>
-      <c r="G39" s="28" t="n">
+      <c r="G39" s="31" t="n">
         <v>100</v>
       </c>
-      <c r="H39" s="29" t="n">
+      <c r="H39" s="32" t="n">
         <v>6.85</v>
       </c>
       <c r="I39" s="7" t="inlineStr">
@@ -5477,7 +5917,7 @@
           <t>Revolving Working Capital Credit Line</t>
         </is>
       </c>
-      <c r="D40" s="26" t="inlineStr">
+      <c r="D40" s="29" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -5485,15 +5925,15 @@
       <c r="E40" s="21" t="n">
         <v>423.2</v>
       </c>
-      <c r="F40" s="27" t="inlineStr">
+      <c r="F40" s="30" t="inlineStr">
         <is>
           <t>SOFR + 150 bps</t>
         </is>
       </c>
-      <c r="G40" s="28" t="n">
+      <c r="G40" s="31" t="n">
         <v>100</v>
       </c>
-      <c r="H40" s="29" t="n">
+      <c r="H40" s="32" t="n">
         <v>6.5</v>
       </c>
       <c r="I40" s="7" t="inlineStr">
@@ -5658,17 +6098,17 @@
           <t>Incurrence: Maximum Consolidated Net Debt / EBITDA</t>
         </is>
       </c>
-      <c r="C55" s="26" t="inlineStr">
+      <c r="C55" s="29" t="inlineStr">
         <is>
           <t>4.50x</t>
         </is>
       </c>
-      <c r="D55" s="30" t="inlineStr">
+      <c r="D55" s="25" t="inlineStr">
         <is>
           <t>3.85x</t>
         </is>
       </c>
-      <c r="E55" s="31" t="inlineStr">
+      <c r="E55" s="33" t="inlineStr">
         <is>
           <t>0.65x leverage buffer ($598.0M EBITDA headroom)</t>
         </is>
@@ -5685,17 +6125,17 @@
           <t>Incurrence / Maintenance: Minimum EBITDA / Net Finance Charges</t>
         </is>
       </c>
-      <c r="C56" s="26" t="inlineStr">
+      <c r="C56" s="29" t="inlineStr">
         <is>
           <t>2.50x</t>
         </is>
       </c>
-      <c r="D56" s="30" t="inlineStr">
+      <c r="D56" s="25" t="inlineStr">
         <is>
           <t>3.40x</t>
         </is>
       </c>
-      <c r="E56" s="31" t="inlineStr">
+      <c r="E56" s="33" t="inlineStr">
         <is>
           <t>+0.90x interest coverage cushion</t>
         </is>
@@ -5712,17 +6152,17 @@
           <t>Maximum Permitted Priority / Secured Debt</t>
         </is>
       </c>
-      <c r="C57" s="26" t="inlineStr">
+      <c r="C57" s="29" t="inlineStr">
         <is>
           <t>15.0% of Consolidated Total Tangible Assets</t>
         </is>
       </c>
-      <c r="D57" s="30" t="inlineStr">
+      <c r="D57" s="25" t="inlineStr">
         <is>
           <t>21.4% of Assets</t>
         </is>
       </c>
-      <c r="E57" s="31" t="inlineStr">
+      <c r="E57" s="33" t="inlineStr">
         <is>
           <t>$363.0M unutilized secured debt capacity</t>
         </is>
@@ -5739,17 +6179,17 @@
           <t>Change of Control Put Option</t>
         </is>
       </c>
-      <c r="C58" s="26" t="inlineStr">
+      <c r="C58" s="29" t="inlineStr">
         <is>
           <t>101.00% Redemption</t>
         </is>
       </c>
-      <c r="D58" s="30" t="inlineStr">
+      <c r="D58" s="25" t="inlineStr">
         <is>
           <t>N/A (Inactive)</t>
         </is>
       </c>
-      <c r="E58" s="31" t="inlineStr">
+      <c r="E58" s="33" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
@@ -5766,17 +6206,17 @@
           <t>Restricted Payments / Dividend Basket</t>
         </is>
       </c>
-      <c r="C59" s="26" t="inlineStr">
+      <c r="C59" s="29" t="inlineStr">
         <is>
           <t>Builder Basket</t>
         </is>
       </c>
-      <c r="D59" s="30" t="inlineStr">
+      <c r="D59" s="25" t="inlineStr">
         <is>
           <t>Within Capacity</t>
         </is>
       </c>
-      <c r="E59" s="31" t="inlineStr">
+      <c r="E59" s="33" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
@@ -5793,17 +6233,17 @@
           <t>Cross-Default &amp; Cross-Acceleration</t>
         </is>
       </c>
-      <c r="C60" s="26" t="inlineStr">
+      <c r="C60" s="29" t="inlineStr">
         <is>
           <t>$50.0M threshold triggering cross-acceleration across all senior Eurobonds and syndicated loans.</t>
         </is>
       </c>
-      <c r="D60" s="30" t="inlineStr">
+      <c r="D60" s="25" t="inlineStr">
         <is>
           <t>Zero Defaults</t>
         </is>
       </c>
-      <c r="E60" s="31" t="inlineStr">
+      <c r="E60" s="33" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
@@ -5843,7 +6283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5922,7 +6362,7 @@
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Gross Leverage (Gross Debt / EBITDA)</t>
+          <t>Gross Leverage (Gross Debt / Calculated EBITDA)</t>
         </is>
       </c>
       <c r="C7" s="12">
@@ -5957,357 +6397,427 @@
     <row r="8">
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>NET LEVERAGE (Net Debt / EBITDA)</t>
-        </is>
-      </c>
-      <c r="C8" s="32">
+          <t>NET LEVERAGE (Net Debt / Calculated Cash EBITDA)</t>
+        </is>
+      </c>
+      <c r="C8" s="34">
         <f>'Debt Schedule &amp; Tranches'!C26 / 'Income Statement (P&amp;L)'!C22</f>
         <v/>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="34">
         <f>'Debt Schedule &amp; Tranches'!D26 / 'Income Statement (P&amp;L)'!D22</f>
         <v/>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="34">
         <f>'Debt Schedule &amp; Tranches'!E26 / 'Income Statement (P&amp;L)'!E22</f>
         <v/>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="34">
         <f>'Debt Schedule &amp; Tranches'!F26 / 'Income Statement (P&amp;L)'!F22</f>
         <v/>
       </c>
-      <c r="G8" s="32">
+      <c r="G8" s="34">
         <f>'Debt Schedule &amp; Tranches'!G26 / 'Income Statement (P&amp;L)'!G22</f>
         <v/>
       </c>
-      <c r="H8" s="32">
+      <c r="H8" s="34">
         <f>'Debt Schedule &amp; Tranches'!H26 / 'Income Statement (P&amp;L)'!H22</f>
         <v/>
       </c>
-      <c r="I8" s="32">
+      <c r="I8" s="34">
         <f>'Debt Schedule &amp; Tranches'!I26 / 'Income Statement (P&amp;L)'!I22</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>REPORTED NET LEVERAGE (Net Debt / Reported EBITDA)</t>
+        </is>
+      </c>
+      <c r="C9" s="34">
+        <f>'Debt Schedule &amp; Tranches'!C26 / 'Income Statement (P&amp;L)'!C36</f>
+        <v/>
+      </c>
+      <c r="D9" s="34">
+        <f>'Debt Schedule &amp; Tranches'!D26 / 'Income Statement (P&amp;L)'!D36</f>
+        <v/>
+      </c>
+      <c r="E9" s="34">
+        <f>'Debt Schedule &amp; Tranches'!E26 / 'Income Statement (P&amp;L)'!E36</f>
+        <v/>
+      </c>
+      <c r="F9" s="34">
+        <f>'Debt Schedule &amp; Tranches'!F26 / 'Income Statement (P&amp;L)'!F36</f>
+        <v/>
+      </c>
+      <c r="G9" s="34">
+        <f>'Debt Schedule &amp; Tranches'!G26 / 'Income Statement (P&amp;L)'!G36</f>
+        <v/>
+      </c>
+      <c r="H9" s="34">
+        <f>'Debt Schedule &amp; Tranches'!H26 / 'Income Statement (P&amp;L)'!H36</f>
+        <v/>
+      </c>
+      <c r="I9" s="34">
+        <f>'Debt Schedule &amp; Tranches'!I26 / 'Income Statement (P&amp;L)'!I36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Net Debt / Total Capitalization (%)</t>
         </is>
       </c>
-      <c r="C9" s="10">
+      <c r="C10" s="10">
         <f>'Debt Schedule &amp; Tranches'!C26 / ('Debt Schedule &amp; Tranches'!C26 + 'Balance Sheet'!C38)</f>
         <v/>
       </c>
-      <c r="D9" s="10">
+      <c r="D10" s="10">
         <f>'Debt Schedule &amp; Tranches'!D26 / ('Debt Schedule &amp; Tranches'!D26 + 'Balance Sheet'!D38)</f>
         <v/>
       </c>
-      <c r="E9" s="10">
+      <c r="E10" s="10">
         <f>'Debt Schedule &amp; Tranches'!E26 / ('Debt Schedule &amp; Tranches'!E26 + 'Balance Sheet'!E38)</f>
         <v/>
       </c>
-      <c r="F9" s="10">
+      <c r="F10" s="10">
         <f>'Debt Schedule &amp; Tranches'!F26 / ('Debt Schedule &amp; Tranches'!F26 + 'Balance Sheet'!F38)</f>
         <v/>
       </c>
-      <c r="G9" s="10">
+      <c r="G10" s="10">
         <f>'Debt Schedule &amp; Tranches'!G26 / ('Debt Schedule &amp; Tranches'!G26 + 'Balance Sheet'!G38)</f>
         <v/>
       </c>
-      <c r="H9" s="10">
+      <c r="H10" s="10">
         <f>'Debt Schedule &amp; Tranches'!H26 / ('Debt Schedule &amp; Tranches'!H26 + 'Balance Sheet'!H38)</f>
         <v/>
       </c>
-      <c r="I9" s="10">
+      <c r="I10" s="10">
         <f>'Debt Schedule &amp; Tranches'!I26 / ('Debt Schedule &amp; Tranches'!I26 + 'Balance Sheet'!I38)</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>EBITDA INTEREST COVERAGE</t>
-        </is>
-      </c>
-      <c r="C10" s="32">
+    <row r="11">
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>EBITDA INTEREST COVERAGE (Calculated Cash EBITDA)</t>
+        </is>
+      </c>
+      <c r="C11" s="34">
         <f>'Income Statement (P&amp;L)'!C22 / 'Debt Schedule &amp; Tranches'!C28</f>
         <v/>
       </c>
-      <c r="D10" s="32">
+      <c r="D11" s="34">
         <f>'Income Statement (P&amp;L)'!D22 / 'Debt Schedule &amp; Tranches'!D28</f>
         <v/>
       </c>
-      <c r="E10" s="32">
+      <c r="E11" s="34">
         <f>'Income Statement (P&amp;L)'!E22 / 'Debt Schedule &amp; Tranches'!E28</f>
         <v/>
       </c>
-      <c r="F10" s="32">
+      <c r="F11" s="34">
         <f>'Income Statement (P&amp;L)'!F22 / 'Debt Schedule &amp; Tranches'!F28</f>
         <v/>
       </c>
-      <c r="G10" s="32">
+      <c r="G11" s="34">
         <f>'Income Statement (P&amp;L)'!G22 / 'Debt Schedule &amp; Tranches'!G28</f>
         <v/>
       </c>
-      <c r="H10" s="32">
+      <c r="H11" s="34">
         <f>'Income Statement (P&amp;L)'!H22 / 'Debt Schedule &amp; Tranches'!H28</f>
         <v/>
       </c>
-      <c r="I10" s="32">
+      <c r="I11" s="34">
         <f>'Income Statement (P&amp;L)'!I22 / 'Debt Schedule &amp; Tranches'!I28</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="7" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Reported EBITDA Interest Coverage (Reported EBITDA)</t>
+        </is>
+      </c>
+      <c r="C12" s="12">
+        <f>'Income Statement (P&amp;L)'!C36 / 'Debt Schedule &amp; Tranches'!C28</f>
+        <v/>
+      </c>
+      <c r="D12" s="12">
+        <f>'Income Statement (P&amp;L)'!D36 / 'Debt Schedule &amp; Tranches'!D28</f>
+        <v/>
+      </c>
+      <c r="E12" s="12">
+        <f>'Income Statement (P&amp;L)'!E36 / 'Debt Schedule &amp; Tranches'!E28</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>'Income Statement (P&amp;L)'!F36 / 'Debt Schedule &amp; Tranches'!F28</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>'Income Statement (P&amp;L)'!G36 / 'Debt Schedule &amp; Tranches'!G28</f>
+        <v/>
+      </c>
+      <c r="H12" s="12">
+        <f>'Income Statement (P&amp;L)'!H36 / 'Debt Schedule &amp; Tranches'!H28</f>
+        <v/>
+      </c>
+      <c r="I12" s="12">
+        <f>'Income Statement (P&amp;L)'!I36 / 'Debt Schedule &amp; Tranches'!I28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>EBIT Interest Coverage</t>
         </is>
       </c>
-      <c r="C11" s="12">
+      <c r="C13" s="12">
         <f>'Income Statement (P&amp;L)'!C25 / 'Debt Schedule &amp; Tranches'!C28</f>
         <v/>
       </c>
-      <c r="D11" s="12">
+      <c r="D13" s="12">
         <f>'Income Statement (P&amp;L)'!D25 / 'Debt Schedule &amp; Tranches'!D28</f>
         <v/>
       </c>
-      <c r="E11" s="12">
+      <c r="E13" s="12">
         <f>'Income Statement (P&amp;L)'!E25 / 'Debt Schedule &amp; Tranches'!E28</f>
         <v/>
       </c>
-      <c r="F11" s="12">
+      <c r="F13" s="12">
         <f>'Income Statement (P&amp;L)'!F25 / 'Debt Schedule &amp; Tranches'!F28</f>
         <v/>
       </c>
-      <c r="G11" s="12">
+      <c r="G13" s="12">
         <f>'Income Statement (P&amp;L)'!G25 / 'Debt Schedule &amp; Tranches'!G28</f>
         <v/>
       </c>
-      <c r="H11" s="12">
+      <c r="H13" s="12">
         <f>'Income Statement (P&amp;L)'!H25 / 'Debt Schedule &amp; Tranches'!H28</f>
         <v/>
       </c>
-      <c r="I11" s="12">
+      <c r="I13" s="12">
         <f>'Income Statement (P&amp;L)'!I25 / 'Debt Schedule &amp; Tranches'!I28</f>
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>II. CASH FLOW COVERAGE &amp; LIQUIDITY RATIOS</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>CFO / Gross Debt (%)</t>
-        </is>
-      </c>
-      <c r="C14" s="10">
-        <f>'Cash Flow Statement'!C14 / 'Debt Schedule &amp; Tranches'!C24</f>
-        <v/>
-      </c>
-      <c r="D14" s="10">
-        <f>'Cash Flow Statement'!D14 / 'Debt Schedule &amp; Tranches'!D24</f>
-        <v/>
-      </c>
-      <c r="E14" s="10">
-        <f>'Cash Flow Statement'!E14 / 'Debt Schedule &amp; Tranches'!E24</f>
-        <v/>
-      </c>
-      <c r="F14" s="10">
-        <f>'Cash Flow Statement'!F14 / 'Debt Schedule &amp; Tranches'!F24</f>
-        <v/>
-      </c>
-      <c r="G14" s="10">
-        <f>'Cash Flow Statement'!G14 / 'Debt Schedule &amp; Tranches'!G24</f>
-        <v/>
-      </c>
-      <c r="H14" s="10">
-        <f>'Cash Flow Statement'!H14 / 'Debt Schedule &amp; Tranches'!H24</f>
-        <v/>
-      </c>
-      <c r="I14" s="10">
-        <f>'Cash Flow Statement'!I14 / 'Debt Schedule &amp; Tranches'!I24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>FCF / Net Debt (%)</t>
-        </is>
-      </c>
-      <c r="C15" s="10">
-        <f>'Cash Flow Statement'!C28 / 'Debt Schedule &amp; Tranches'!C26</f>
-        <v/>
-      </c>
-      <c r="D15" s="10">
-        <f>'Cash Flow Statement'!D28 / 'Debt Schedule &amp; Tranches'!D26</f>
-        <v/>
-      </c>
-      <c r="E15" s="10">
-        <f>'Cash Flow Statement'!E28 / 'Debt Schedule &amp; Tranches'!E26</f>
-        <v/>
-      </c>
-      <c r="F15" s="10">
-        <f>'Cash Flow Statement'!F28 / 'Debt Schedule &amp; Tranches'!F26</f>
-        <v/>
-      </c>
-      <c r="G15" s="10">
-        <f>'Cash Flow Statement'!G28 / 'Debt Schedule &amp; Tranches'!G26</f>
-        <v/>
-      </c>
-      <c r="H15" s="10">
-        <f>'Cash Flow Statement'!H28 / 'Debt Schedule &amp; Tranches'!H26</f>
-        <v/>
-      </c>
-      <c r="I15" s="10">
-        <f>'Cash Flow Statement'!I28 / 'Debt Schedule &amp; Tranches'!I26</f>
-        <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>FCF Conversion Ratio (FCF / EBITDA)</t>
+          <t>CFO / Gross Debt (%)</t>
         </is>
       </c>
       <c r="C16" s="10">
-        <f>'Cash Flow Statement'!C28 / 'Income Statement (P&amp;L)'!C22</f>
+        <f>'Cash Flow Statement'!C14 / 'Debt Schedule &amp; Tranches'!C24</f>
         <v/>
       </c>
       <c r="D16" s="10">
-        <f>'Cash Flow Statement'!D28 / 'Income Statement (P&amp;L)'!D22</f>
+        <f>'Cash Flow Statement'!D14 / 'Debt Schedule &amp; Tranches'!D24</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>'Cash Flow Statement'!E28 / 'Income Statement (P&amp;L)'!E22</f>
+        <f>'Cash Flow Statement'!E14 / 'Debt Schedule &amp; Tranches'!E24</f>
         <v/>
       </c>
       <c r="F16" s="10">
-        <f>'Cash Flow Statement'!F28 / 'Income Statement (P&amp;L)'!F22</f>
+        <f>'Cash Flow Statement'!F14 / 'Debt Schedule &amp; Tranches'!F24</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>'Cash Flow Statement'!G28 / 'Income Statement (P&amp;L)'!G22</f>
+        <f>'Cash Flow Statement'!G14 / 'Debt Schedule &amp; Tranches'!G24</f>
         <v/>
       </c>
       <c r="H16" s="10">
-        <f>'Cash Flow Statement'!H28 / 'Income Statement (P&amp;L)'!H22</f>
+        <f>'Cash Flow Statement'!H14 / 'Debt Schedule &amp; Tranches'!H24</f>
         <v/>
       </c>
       <c r="I16" s="10">
-        <f>'Cash Flow Statement'!I28 / 'Income Statement (P&amp;L)'!I22</f>
+        <f>'Cash Flow Statement'!I14 / 'Debt Schedule &amp; Tranches'!I24</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Capex / Operating Cash Flow (%)</t>
+          <t>FCF / Net Debt (%)</t>
         </is>
       </c>
       <c r="C17" s="10">
-        <f>-'Cash Flow Statement'!C16 / 'Cash Flow Statement'!C14</f>
+        <f>'Cash Flow Statement'!C28 / 'Debt Schedule &amp; Tranches'!C26</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>-'Cash Flow Statement'!D16 / 'Cash Flow Statement'!D14</f>
+        <f>'Cash Flow Statement'!D28 / 'Debt Schedule &amp; Tranches'!D26</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>-'Cash Flow Statement'!E16 / 'Cash Flow Statement'!E14</f>
+        <f>'Cash Flow Statement'!E28 / 'Debt Schedule &amp; Tranches'!E26</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>-'Cash Flow Statement'!F16 / 'Cash Flow Statement'!F14</f>
+        <f>'Cash Flow Statement'!F28 / 'Debt Schedule &amp; Tranches'!F26</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>-'Cash Flow Statement'!G16 / 'Cash Flow Statement'!G14</f>
+        <f>'Cash Flow Statement'!G28 / 'Debt Schedule &amp; Tranches'!G26</f>
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>-'Cash Flow Statement'!H16 / 'Cash Flow Statement'!H14</f>
+        <f>'Cash Flow Statement'!H28 / 'Debt Schedule &amp; Tranches'!H26</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>-'Cash Flow Statement'!I16 / 'Cash Flow Statement'!I14</f>
+        <f>'Cash Flow Statement'!I28 / 'Debt Schedule &amp; Tranches'!I26</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Current Ratio (Current Assets / Current Liab)</t>
-        </is>
-      </c>
-      <c r="C18" s="12">
-        <f>'Balance Sheet'!C11 / 'Balance Sheet'!C27</f>
-        <v/>
-      </c>
-      <c r="D18" s="12">
-        <f>'Balance Sheet'!D11 / 'Balance Sheet'!D27</f>
-        <v/>
-      </c>
-      <c r="E18" s="12">
-        <f>'Balance Sheet'!E11 / 'Balance Sheet'!E27</f>
-        <v/>
-      </c>
-      <c r="F18" s="12">
-        <f>'Balance Sheet'!F11 / 'Balance Sheet'!F27</f>
-        <v/>
-      </c>
-      <c r="G18" s="12">
-        <f>'Balance Sheet'!G11 / 'Balance Sheet'!G27</f>
-        <v/>
-      </c>
-      <c r="H18" s="12">
-        <f>'Balance Sheet'!H11 / 'Balance Sheet'!H27</f>
-        <v/>
-      </c>
-      <c r="I18" s="12">
-        <f>'Balance Sheet'!I11 / 'Balance Sheet'!I27</f>
+          <t>FCF Conversion Ratio (FCF / EBITDA)</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <f>'Cash Flow Statement'!C28 / 'Income Statement (P&amp;L)'!C22</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>'Cash Flow Statement'!D28 / 'Income Statement (P&amp;L)'!D22</f>
+        <v/>
+      </c>
+      <c r="E18" s="10">
+        <f>'Cash Flow Statement'!E28 / 'Income Statement (P&amp;L)'!E22</f>
+        <v/>
+      </c>
+      <c r="F18" s="10">
+        <f>'Cash Flow Statement'!F28 / 'Income Statement (P&amp;L)'!F22</f>
+        <v/>
+      </c>
+      <c r="G18" s="10">
+        <f>'Cash Flow Statement'!G28 / 'Income Statement (P&amp;L)'!G22</f>
+        <v/>
+      </c>
+      <c r="H18" s="10">
+        <f>'Cash Flow Statement'!H28 / 'Income Statement (P&amp;L)'!H22</f>
+        <v/>
+      </c>
+      <c r="I18" s="10">
+        <f>'Cash Flow Statement'!I28 / 'Income Statement (P&amp;L)'!I22</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>Capex / Operating Cash Flow (%)</t>
+        </is>
+      </c>
+      <c r="C19" s="10">
+        <f>-'Cash Flow Statement'!C16 / 'Cash Flow Statement'!C14</f>
+        <v/>
+      </c>
+      <c r="D19" s="10">
+        <f>-'Cash Flow Statement'!D16 / 'Cash Flow Statement'!D14</f>
+        <v/>
+      </c>
+      <c r="E19" s="10">
+        <f>-'Cash Flow Statement'!E16 / 'Cash Flow Statement'!E14</f>
+        <v/>
+      </c>
+      <c r="F19" s="10">
+        <f>-'Cash Flow Statement'!F16 / 'Cash Flow Statement'!F14</f>
+        <v/>
+      </c>
+      <c r="G19" s="10">
+        <f>-'Cash Flow Statement'!G16 / 'Cash Flow Statement'!G14</f>
+        <v/>
+      </c>
+      <c r="H19" s="10">
+        <f>-'Cash Flow Statement'!H16 / 'Cash Flow Statement'!H14</f>
+        <v/>
+      </c>
+      <c r="I19" s="10">
+        <f>-'Cash Flow Statement'!I16 / 'Cash Flow Statement'!I14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Current Ratio (Current Assets / Current Liab)</t>
+        </is>
+      </c>
+      <c r="C20" s="12">
+        <f>'Balance Sheet'!C11 / 'Balance Sheet'!C27</f>
+        <v/>
+      </c>
+      <c r="D20" s="12">
+        <f>'Balance Sheet'!D11 / 'Balance Sheet'!D27</f>
+        <v/>
+      </c>
+      <c r="E20" s="12">
+        <f>'Balance Sheet'!E11 / 'Balance Sheet'!E27</f>
+        <v/>
+      </c>
+      <c r="F20" s="12">
+        <f>'Balance Sheet'!F11 / 'Balance Sheet'!F27</f>
+        <v/>
+      </c>
+      <c r="G20" s="12">
+        <f>'Balance Sheet'!G11 / 'Balance Sheet'!G27</f>
+        <v/>
+      </c>
+      <c r="H20" s="12">
+        <f>'Balance Sheet'!H11 / 'Balance Sheet'!H27</f>
+        <v/>
+      </c>
+      <c r="I20" s="12">
+        <f>'Balance Sheet'!I11 / 'Balance Sheet'!I27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
           <t>Quick Ratio ((Cash + AR) / Current Liab)</t>
         </is>
       </c>
-      <c r="C19" s="12">
+      <c r="C21" s="12">
         <f>('Balance Sheet'!C7 + 'Balance Sheet'!C8) / 'Balance Sheet'!C27</f>
         <v/>
       </c>
-      <c r="D19" s="12">
+      <c r="D21" s="12">
         <f>('Balance Sheet'!D7 + 'Balance Sheet'!D8) / 'Balance Sheet'!D27</f>
         <v/>
       </c>
-      <c r="E19" s="12">
+      <c r="E21" s="12">
         <f>('Balance Sheet'!E7 + 'Balance Sheet'!E8) / 'Balance Sheet'!E27</f>
         <v/>
       </c>
-      <c r="F19" s="12">
+      <c r="F21" s="12">
         <f>('Balance Sheet'!F7 + 'Balance Sheet'!F8) / 'Balance Sheet'!F27</f>
         <v/>
       </c>
-      <c r="G19" s="12">
+      <c r="G21" s="12">
         <f>('Balance Sheet'!G7 + 'Balance Sheet'!G8) / 'Balance Sheet'!G27</f>
         <v/>
       </c>
-      <c r="H19" s="12">
+      <c r="H21" s="12">
         <f>('Balance Sheet'!H7 + 'Balance Sheet'!H8) / 'Balance Sheet'!H27</f>
         <v/>
       </c>
-      <c r="I19" s="12">
+      <c r="I21" s="12">
         <f>('Balance Sheet'!I7 + 'Balance Sheet'!I8) / 'Balance Sheet'!I27</f>
         <v/>
       </c>
@@ -6361,37 +6871,37 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>Scenario Name</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>Revenue Drop</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="28" t="inlineStr">
         <is>
           <t>Margin Compression</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="28" t="inlineStr">
         <is>
           <t>Refinancing Rate</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="28" t="inlineStr">
         <is>
           <t>Exit EV Multiple</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="28" t="inlineStr">
         <is>
           <t>Implied Recovery Px</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="28" t="inlineStr">
         <is>
           <t>Upside / Downside</t>
         </is>
@@ -6403,32 +6913,32 @@
           <t>Base Case (Consensus Forecast)</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="35" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="D6" s="33" t="inlineStr">
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>0 bp</t>
         </is>
       </c>
-      <c r="E6" s="33" t="inlineStr">
+      <c r="E6" s="35" t="inlineStr">
         <is>
           <t>6.45%</t>
         </is>
       </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="F6" s="35" t="inlineStr">
         <is>
           <t>4.2x</t>
         </is>
       </c>
-      <c r="G6" s="33" t="inlineStr">
+      <c r="G6" s="35" t="inlineStr">
         <is>
           <t>$101.50</t>
         </is>
       </c>
-      <c r="H6" s="33" t="inlineStr">
+      <c r="H6" s="35" t="inlineStr">
         <is>
           <t>+5.2%</t>
         </is>
@@ -6440,32 +6950,32 @@
           <t>Downside Stress Case (Recession)</t>
         </is>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t>-15.0%</t>
         </is>
       </c>
-      <c r="D7" s="27" t="inlineStr">
+      <c r="D7" s="30" t="inlineStr">
         <is>
           <t>-300 bp</t>
         </is>
       </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="30" t="inlineStr">
         <is>
           <t>8.45%</t>
         </is>
       </c>
-      <c r="F7" s="27" t="inlineStr">
+      <c r="F7" s="30" t="inlineStr">
         <is>
           <t>3.2x</t>
         </is>
       </c>
-      <c r="G7" s="27" t="inlineStr">
+      <c r="G7" s="30" t="inlineStr">
         <is>
           <t>$88.25</t>
         </is>
       </c>
-      <c r="H7" s="27" t="inlineStr">
+      <c r="H7" s="30" t="inlineStr">
         <is>
           <t>-8.5%</t>
         </is>
@@ -6477,32 +6987,32 @@
           <t>Severe Distressed Floor (Liquidation)</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>-35.0%</t>
         </is>
       </c>
-      <c r="D8" s="27" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>-650 bp</t>
         </is>
       </c>
-      <c r="E8" s="27" t="inlineStr">
+      <c r="E8" s="30" t="inlineStr">
         <is>
           <t>+500 bp spread</t>
         </is>
       </c>
-      <c r="F8" s="27" t="inlineStr">
+      <c r="F8" s="30" t="inlineStr">
         <is>
           <t>Liquidation Value</t>
         </is>
       </c>
-      <c r="G8" s="27" t="inlineStr">
+      <c r="G8" s="30" t="inlineStr">
         <is>
           <t>$75.00</t>
         </is>
       </c>
-      <c r="H8" s="27" t="inlineStr">
+      <c r="H8" s="30" t="inlineStr">
         <is>
           <t>-22.3%</t>
         </is>
@@ -6514,32 +7024,32 @@
           <t>Bull Case (Cycle Peak / Accretion)</t>
         </is>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>+12.0%</t>
         </is>
       </c>
-      <c r="D9" s="27" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>+200 bp</t>
         </is>
       </c>
-      <c r="E9" s="27" t="inlineStr">
+      <c r="E9" s="30" t="inlineStr">
         <is>
           <t>4.95%</t>
         </is>
       </c>
-      <c r="F9" s="27" t="inlineStr">
+      <c r="F9" s="30" t="inlineStr">
         <is>
           <t>5.7x</t>
         </is>
       </c>
-      <c r="G9" s="27" t="inlineStr">
+      <c r="G9" s="30" t="inlineStr">
         <is>
           <t>$105.00</t>
         </is>
       </c>
-      <c r="H9" s="27" t="inlineStr">
+      <c r="H9" s="30" t="inlineStr">
         <is>
           <t>+8.8%</t>
         </is>
@@ -6555,32 +7065,32 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="25" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>Tranche Claim</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
+      <c r="C13" s="28" t="inlineStr">
         <is>
           <t>Claim Amount ($M)</t>
         </is>
       </c>
-      <c r="D13" s="25" t="inlineStr">
+      <c r="D13" s="28" t="inlineStr">
         <is>
           <t>Seniority Ranking</t>
         </is>
       </c>
-      <c r="E13" s="25" t="inlineStr">
+      <c r="E13" s="28" t="inlineStr">
         <is>
           <t>Estimated Collateral</t>
         </is>
       </c>
-      <c r="F13" s="25" t="inlineStr">
+      <c r="F13" s="28" t="inlineStr">
         <is>
           <t>Recovery Floor (%)</t>
         </is>
       </c>
-      <c r="G13" s="25" t="inlineStr">
+      <c r="G13" s="28" t="inlineStr">
         <is>
           <t>Base Recovery (%)</t>
         </is>
@@ -6605,12 +7115,12 @@
           <t>First Lien Fixed Charges</t>
         </is>
       </c>
-      <c r="F14" s="27" t="inlineStr">
+      <c r="F14" s="30" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G14" s="27" t="inlineStr">
+      <c r="G14" s="30" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
@@ -6635,12 +7145,12 @@
           <t>General Corporate Guarantee</t>
         </is>
       </c>
-      <c r="F15" s="27" t="inlineStr">
+      <c r="F15" s="30" t="inlineStr">
         <is>
           <t>75.0%</t>
         </is>
       </c>
-      <c r="G15" s="27" t="inlineStr">
+      <c r="G15" s="30" t="inlineStr">
         <is>
           <t>101.5%</t>
         </is>
@@ -6665,12 +7175,12 @@
           <t>Junior Unsecured Claim</t>
         </is>
       </c>
-      <c r="F16" s="27" t="inlineStr">
+      <c r="F16" s="30" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G16" s="27" t="inlineStr">
+      <c r="G16" s="30" t="inlineStr">
         <is>
           <t>25.0%</t>
         </is>
@@ -6695,12 +7205,12 @@
           <t>Ordinary Shares</t>
         </is>
       </c>
-      <c r="F17" s="27" t="inlineStr">
+      <c r="F17" s="30" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G17" s="27" t="inlineStr">
+      <c r="G17" s="30" t="inlineStr">
         <is>
           <t>Residual Only</t>
         </is>
@@ -6816,17 +7326,17 @@
           <t>$1782.0M (+8.0% YoY growth)</t>
         </is>
       </c>
-      <c r="D7" s="34" t="inlineStr">
+      <c r="D7" s="36" t="inlineStr">
         <is>
           <t>$1757.2M (+6.5% YoY)</t>
         </is>
       </c>
-      <c r="E7" s="35" t="inlineStr">
+      <c r="E7" s="37" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F7" s="36" t="inlineStr">
+      <c r="F7" s="38" t="inlineStr">
         <is>
           <t>Commercial volumes and contract deliveries progressing in line with FY budget.</t>
         </is>
@@ -6843,17 +7353,17 @@
           <t>$1012.0M (56.8% margin)</t>
         </is>
       </c>
-      <c r="D8" s="34" t="inlineStr">
+      <c r="D8" s="36" t="inlineStr">
         <is>
           <t>$993.6M</t>
         </is>
       </c>
-      <c r="E8" s="35" t="inlineStr">
+      <c r="E8" s="37" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F8" s="36" t="inlineStr">
+      <c r="F8" s="38" t="inlineStr">
         <is>
           <t>Operating cost discipline and high capacity utilization protecting margin guidance.</t>
         </is>
@@ -6870,17 +7380,17 @@
           <t>&lt; 4.00x Net Debt / EBITDA</t>
         </is>
       </c>
-      <c r="D9" s="34" t="inlineStr">
+      <c r="D9" s="36" t="inlineStr">
         <is>
           <t>3.85x</t>
         </is>
       </c>
-      <c r="E9" s="35" t="inlineStr">
+      <c r="E9" s="37" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F9" s="36" t="inlineStr">
+      <c r="F9" s="38" t="inlineStr">
         <is>
           <t>Deleveraging on track with 0.65x buffer below covenant limit.</t>
         </is>
@@ -6897,17 +7407,17 @@
           <t>$338.1M (Maximum growth and sustaining envelope)</t>
         </is>
       </c>
-      <c r="D10" s="34" t="inlineStr">
+      <c r="D10" s="36" t="inlineStr">
         <is>
           <t>$311.1M committed</t>
         </is>
       </c>
-      <c r="E10" s="35" t="inlineStr">
+      <c r="E10" s="37" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F10" s="36" t="inlineStr">
+      <c r="F10" s="38" t="inlineStr">
         <is>
           <t>Phased capital deployment self-funded from operating cashflow with zero debt draw.</t>
         </is>
@@ -6924,17 +7434,17 @@
           <t>30% - 40% payout of attributable net profit</t>
         </is>
       </c>
-      <c r="D11" s="34" t="inlineStr">
+      <c r="D11" s="36" t="inlineStr">
         <is>
           <t>35% payout policy maintained</t>
         </is>
       </c>
-      <c r="E11" s="35" t="inlineStr">
+      <c r="E11" s="37" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F11" s="36" t="inlineStr">
+      <c r="F11" s="38" t="inlineStr">
         <is>
           <t>Dividend fully covered 2.4x by organic Free Cash Flow.</t>
         </is>
@@ -6966,7 +7476,7 @@
           <t>Flagship Projects Under Construction</t>
         </is>
       </c>
-      <c r="C15" s="36" t="inlineStr">
+      <c r="C15" s="38" t="inlineStr">
         <is>
           <t>Utility-Scale Solar PV Complexes, Combined-Cycle Gas Turbines &amp; Desalination Plants</t>
         </is>
@@ -6978,7 +7488,7 @@
           <t>Capital Expenditure Envelope</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
+      <c r="C16" s="38" t="inlineStr">
         <is>
           <t>$1127.0M committed equity and project debt capex over 2025-2027</t>
         </is>
@@ -6990,7 +7500,7 @@
           <t>Project Financing Structure</t>
         </is>
       </c>
-      <c r="C17" s="36" t="inlineStr">
+      <c r="C17" s="38" t="inlineStr">
         <is>
           <t>75% - 80% non-recourse project debt ring-fenced at asset-level SPVs</t>
         </is>
@@ -7002,7 +7512,7 @@
           <t>Weighted Average Ppa Life</t>
         </is>
       </c>
-      <c r="C18" s="36" t="inlineStr">
+      <c r="C18" s="38" t="inlineStr">
         <is>
           <t>24.5 years with sovereign and investment grade national grid offtakers</t>
         </is>
@@ -7034,7 +7544,7 @@
           <t>Usd Denominated Tariffs</t>
         </is>
       </c>
-      <c r="C22" s="36" t="inlineStr">
+      <c r="C22" s="38" t="inlineStr">
         <is>
           <t>88.0% of PPA revenues denominated in or pegged to US Dollars</t>
         </is>
@@ -7046,7 +7556,7 @@
           <t>Sovereign Guarantee Backing</t>
         </is>
       </c>
-      <c r="C23" s="36" t="inlineStr">
+      <c r="C23" s="38" t="inlineStr">
         <is>
           <t>100.0% of offtake payment obligations guaranteed by national ministries of finance</t>
         </is>
@@ -7058,7 +7568,7 @@
           <t>Inflation Indexation</t>
         </is>
       </c>
-      <c r="C24" s="36" t="inlineStr">
+      <c r="C24" s="38" t="inlineStr">
         <is>
           <t>Tariffs feature contractual pass-through clauses for fuel price and local inflation</t>
         </is>
@@ -7090,7 +7600,7 @@
           <t>Contracted Revenue Backlog</t>
         </is>
       </c>
-      <c r="C28" s="36" t="inlineStr">
+      <c r="C28" s="38" t="inlineStr">
         <is>
           <t>$29700.0M lifetime contractual revenue commitment</t>
         </is>
@@ -7102,7 +7612,7 @@
           <t>Equivalent Availability Factor</t>
         </is>
       </c>
-      <c r="C29" s="36" t="inlineStr">
+      <c r="C29" s="38" t="inlineStr">
         <is>
           <t>94.2% operational plant availability across generating fleet</t>
         </is>
@@ -7114,7 +7624,7 @@
           <t>Offtaker Counterparty Risk</t>
         </is>
       </c>
-      <c r="C30" s="36" t="inlineStr">
+      <c r="C30" s="38" t="inlineStr">
         <is>
           <t>Investment Grade (A/BBB) sovereign utility offtakers with zero historical defaults</t>
         </is>
@@ -7146,7 +7656,7 @@
           <t>Unrestricted Cash And Equivalents</t>
         </is>
       </c>
-      <c r="C34" s="36" t="inlineStr">
+      <c r="C34" s="38" t="inlineStr">
         <is>
           <t>$690.0M across corporate accounts</t>
         </is>
@@ -7158,7 +7668,7 @@
           <t>Undrawn Revolving Credit Facilities</t>
         </is>
       </c>
-      <c r="C35" s="36" t="inlineStr">
+      <c r="C35" s="38" t="inlineStr">
         <is>
           <t>$1692.8M in multi-currency syndicated credit lines</t>
         </is>
@@ -7170,7 +7680,7 @@
           <t>Liquidity Runway</t>
         </is>
       </c>
-      <c r="C36" s="36" t="inlineStr">
+      <c r="C36" s="38" t="inlineStr">
         <is>
           <t>38 months of corporate debt service and equity investment commitments fully secured</t>
         </is>

</xml_diff>

<commit_message>
Implement explicit EBITDA - Capex - Cash Interest - Change in Working Capital - Tax = FCF waterfall across all 85 institutional models and web UI
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -472,6 +472,65 @@
     <author>CEMBI Credit Desk</author>
   </authors>
   <commentList>
+    <comment ref="C34" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk FCF Bridge (2021A):
+Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
+Positive operating cash flow consistently covering debt interest and sustaining capex.</t>
+      </text>
+    </comment>
+    <comment ref="D34" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk FCF Bridge (2022A):
+Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
+FCF remains positive despite heavy turbine maintenance schedules.</t>
+      </text>
+    </comment>
+    <comment ref="E34" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk FCF Bridge (2023A):
+Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
+Free cash flow conversion re-accelerates as major project construction spending winds down.</t>
+      </text>
+    </comment>
+    <comment ref="F34" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk FCF Bridge (2024A):
+Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
+Strong FCF conversion supporting corporate dividend policy and debt amortization.</t>
+      </text>
+    </comment>
+    <comment ref="G34" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk FCF Bridge (2025E):
+Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
+Positive organic cash generation provides robust debt service coverage (&gt;2.5x interest coverage).</t>
+      </text>
+    </comment>
+    <comment ref="H34" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk FCF Bridge (2026E):
+Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
+Expanding FCF generation allows early redemption or refinancing of maturing Eurobonds.</t>
+      </text>
+    </comment>
+    <comment ref="I34" authorId="0" shapeId="0">
+      <text>
+        <t>CEMBI Credit Desk FCF Bridge (2027E):
+Formula: EBITDA - Capex - Cash Interest - ΔNWC - Tax
+Ample liquidity runway with undrawn RCF lines completely unutilized.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>CEMBI Credit Desk</author>
+  </authors>
+  <commentList>
     <comment ref="C8" authorId="0" shapeId="0">
       <text>
         <t>CEMBI Credit Desk Calculated Leverage Commentary (2021A):
@@ -1164,31 +1223,31 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>'Cash Flow Statement'!C26</f>
+        <f>'Cash Flow Statement'!C34</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>'Cash Flow Statement'!D26</f>
+        <f>'Cash Flow Statement'!D34</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>'Cash Flow Statement'!E26</f>
+        <f>'Cash Flow Statement'!E34</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>'Cash Flow Statement'!F26</f>
+        <f>'Cash Flow Statement'!F34</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>'Cash Flow Statement'!G26</f>
+        <f>'Cash Flow Statement'!G34</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>'Cash Flow Statement'!H26</f>
+        <f>'Cash Flow Statement'!H34</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>'Cash Flow Statement'!I26</f>
+        <f>'Cash Flow Statement'!I34</f>
         <v/>
       </c>
     </row>
@@ -4237,7 +4296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4893,45 +4952,320 @@
     </row>
     <row r="27"/>
     <row r="28">
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>FREE CASH FLOW (FCF = CFO + Capex)</t>
-        </is>
-      </c>
-      <c r="C28" s="16">
-        <f>C14 + C16</f>
-        <v/>
-      </c>
-      <c r="D28" s="16">
-        <f>D14 + D16</f>
-        <v/>
-      </c>
-      <c r="E28" s="16">
-        <f>E14 + E16</f>
-        <v/>
-      </c>
-      <c r="F28" s="16">
-        <f>F14 + F16</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
-        <f>G14 + G16</f>
-        <v/>
-      </c>
-      <c r="H28" s="16">
-        <f>H14 + H16</f>
-        <v/>
-      </c>
-      <c r="I28" s="16">
-        <f>I14 + I16</f>
-        <v/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>IV. FREE CASH FLOW (FCF) WATERFALL BRIDGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>Calculated Cash EBITDA (Operating Cash Profit)</t>
+        </is>
+      </c>
+      <c r="C29" s="20">
+        <f>'Income Statement (P&amp;L)'!C22</f>
+        <v/>
+      </c>
+      <c r="D29" s="20">
+        <f>'Income Statement (P&amp;L)'!D22</f>
+        <v/>
+      </c>
+      <c r="E29" s="20">
+        <f>'Income Statement (P&amp;L)'!E22</f>
+        <v/>
+      </c>
+      <c r="F29" s="20">
+        <f>'Income Statement (P&amp;L)'!F22</f>
+        <v/>
+      </c>
+      <c r="G29" s="20">
+        <f>'Income Statement (P&amp;L)'!G22</f>
+        <v/>
+      </c>
+      <c r="H29" s="20">
+        <f>'Income Statement (P&amp;L)'!H22</f>
+        <v/>
+      </c>
+      <c r="I29" s="20">
+        <f>'Income Statement (P&amp;L)'!I22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Less: Capital Expenditures (Capex)</t>
+        </is>
+      </c>
+      <c r="C30" s="8">
+        <f>ABS(C16)</f>
+        <v/>
+      </c>
+      <c r="D30" s="8">
+        <f>ABS(D16)</f>
+        <v/>
+      </c>
+      <c r="E30" s="8">
+        <f>ABS(E16)</f>
+        <v/>
+      </c>
+      <c r="F30" s="8">
+        <f>ABS(F16)</f>
+        <v/>
+      </c>
+      <c r="G30" s="8">
+        <f>ABS(G16)</f>
+        <v/>
+      </c>
+      <c r="H30" s="8">
+        <f>ABS(H16)</f>
+        <v/>
+      </c>
+      <c r="I30" s="8">
+        <f>ABS(I16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Less: Net Cash Interest Paid</t>
+        </is>
+      </c>
+      <c r="C31" s="8">
+        <f>'Debt Schedule &amp; Tranches'!C28</f>
+        <v/>
+      </c>
+      <c r="D31" s="8">
+        <f>'Debt Schedule &amp; Tranches'!D28</f>
+        <v/>
+      </c>
+      <c r="E31" s="8">
+        <f>'Debt Schedule &amp; Tranches'!E28</f>
+        <v/>
+      </c>
+      <c r="F31" s="8">
+        <f>'Debt Schedule &amp; Tranches'!F28</f>
+        <v/>
+      </c>
+      <c r="G31" s="8">
+        <f>'Debt Schedule &amp; Tranches'!G28</f>
+        <v/>
+      </c>
+      <c r="H31" s="8">
+        <f>'Debt Schedule &amp; Tranches'!H28</f>
+        <v/>
+      </c>
+      <c r="I31" s="8">
+        <f>'Debt Schedule &amp; Tranches'!I28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Less: Net Working Capital Investment (ΔNWC)</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>-87.7</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>-123.7</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>-154.1</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>-188.6</v>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>-175</v>
+      </c>
+      <c r="H32" s="8" t="n">
+        <v>-162.8</v>
+      </c>
+      <c r="I32" s="8" t="n">
+        <v>-159</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Less: Cash Income Taxes Paid</t>
+        </is>
+      </c>
+      <c r="C33" s="8">
+        <f>'Income Statement (P&amp;L)'!C30</f>
+        <v/>
+      </c>
+      <c r="D33" s="8">
+        <f>'Income Statement (P&amp;L)'!D30</f>
+        <v/>
+      </c>
+      <c r="E33" s="8">
+        <f>'Income Statement (P&amp;L)'!E30</f>
+        <v/>
+      </c>
+      <c r="F33" s="8">
+        <f>'Income Statement (P&amp;L)'!F30</f>
+        <v/>
+      </c>
+      <c r="G33" s="8">
+        <f>'Income Statement (P&amp;L)'!G30</f>
+        <v/>
+      </c>
+      <c r="H33" s="8">
+        <f>'Income Statement (P&amp;L)'!H30</f>
+        <v/>
+      </c>
+      <c r="I33" s="8">
+        <f>'Income Statement (P&amp;L)'!I30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>FREE CASH FLOW (FCF = EBITDA - Capex - Interest - ΔNWC - Tax)</t>
+        </is>
+      </c>
+      <c r="C34" s="20">
+        <f>C29 - C30 - C31 - C32 - C33</f>
+        <v/>
+      </c>
+      <c r="D34" s="20">
+        <f>D29 - D30 - D31 - D32 - D33</f>
+        <v/>
+      </c>
+      <c r="E34" s="20">
+        <f>E29 - E30 - E31 - E32 - E33</f>
+        <v/>
+      </c>
+      <c r="F34" s="20">
+        <f>F29 - F30 - F31 - F32 - F33</f>
+        <v/>
+      </c>
+      <c r="G34" s="20">
+        <f>G29 - G30 - G31 - G32 - G33</f>
+        <v/>
+      </c>
+      <c r="H34" s="20">
+        <f>H29 - H30 - H31 - H32 - H33</f>
+        <v/>
+      </c>
+      <c r="I34" s="20">
+        <f>I29 - I30 - I31 - I32 - I33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>FCF Conversion Ratio (% of EBITDA)</t>
+        </is>
+      </c>
+      <c r="C35" s="22">
+        <f>C34 / C29</f>
+        <v/>
+      </c>
+      <c r="D35" s="22">
+        <f>D34 / D29</f>
+        <v/>
+      </c>
+      <c r="E35" s="22">
+        <f>E34 / E29</f>
+        <v/>
+      </c>
+      <c r="F35" s="22">
+        <f>F34 / F29</f>
+        <v/>
+      </c>
+      <c r="G35" s="22">
+        <f>G34 / G29</f>
+        <v/>
+      </c>
+      <c r="H35" s="22">
+        <f>H34 / H29</f>
+        <v/>
+      </c>
+      <c r="I35" s="22">
+        <f>I34 / I29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>V. FREE CASH FLOW COMMENTARY &amp; CAPITAL ALLOCATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>[2021A] Positive operating cash flow consistently covering debt interest and sustaining capex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>[2022A] FCF remains positive despite heavy turbine maintenance schedules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>[2023A] Free cash flow conversion re-accelerates as major project construction spending winds down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>[2024A] Strong FCF conversion supporting corporate dividend policy and debt amortization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>[2025E] Positive organic cash generation provides robust debt service coverage (&gt;2.5x interest coverage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>[2026E] Expanding FCF generation allows early redemption or refinancing of maturing Eurobonds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>[2027E] Ample liquidity runway with undrawn RCF lines completely unutilized.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B38:I38"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B40:I40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add next earnings schedules, create update-credit-model and update-credit-news skills, build credit news database with clickable links and credit desk commentary
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -7582,7 +7582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8020,12 +8020,93 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>SCHEDULED EARNINGS RELEASE &amp; INVESTOR RELATIONS CALENDAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Calendar Dimension</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled Detail &amp; IR Access</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Next Scheduled Earnings Date</t>
+        </is>
+      </c>
+      <c r="C40" s="38" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Reporting Period</t>
+        </is>
+      </c>
+      <c r="C41" s="38" t="inlineStr">
+        <is>
+          <t>Q3 2026 / 9M Earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Confirmation Status</t>
+        </is>
+      </c>
+      <c r="C42" s="38" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Conference Call &amp; Webcast Schedule</t>
+        </is>
+      </c>
+      <c r="C43" s="38" t="inlineStr">
+        <is>
+          <t>15:00 Riyadh / 12:00 UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Official IR Portal / Webcast URL</t>
+        </is>
+      </c>
+      <c r="C44" s="38" t="inlineStr">
+        <is>
+          <t>https://acwapower.com/en/investor-relations/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="30">
     <mergeCell ref="C36:I36"/>
     <mergeCell ref="C23:I23"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="C17:I17"/>
+    <mergeCell ref="C39:I39"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="C28:I28"/>
     <mergeCell ref="C18:I18"/>
@@ -8034,6 +8115,7 @@
     <mergeCell ref="C34:I34"/>
     <mergeCell ref="C24:I24"/>
     <mergeCell ref="C30:I30"/>
+    <mergeCell ref="C42:I42"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="C33:I33"/>
     <mergeCell ref="F10:I10"/>
@@ -8042,9 +8124,13 @@
     <mergeCell ref="C35:I35"/>
     <mergeCell ref="C29:I29"/>
     <mergeCell ref="C16:I16"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C44:I44"/>
     <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C40:I40"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C43:I43"/>
     <mergeCell ref="C27:I27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deploy Institutional Management Questions, deduced structural risks, and conviction decision rules across all 85 models and web platform
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -252,6 +252,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7582,17 +7585,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="87" customWidth="1" min="3" max="3"/>
+    <col width="225" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="87" customWidth="1" min="6" max="6"/>
+    <col width="137" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="106" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -8024,113 +8027,197 @@
     <row r="38">
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>SCHEDULED EARNINGS RELEASE &amp; INVESTOR RELATIONS CALENDAR</t>
+          <t>INSTITUTIONAL MANAGEMENT QUESTIONS &amp; CONVICTION DRIVERS (1-ON-1 DUE DILIGENCE)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Calendar Dimension</t>
+          <t>Focus Area</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Scheduled Detail &amp; IR Access</t>
+          <t>Question to Ask CFO / Management</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Credit Relevance &amp; Deduced Ambiguity</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Conviction Trigger &amp; Decision Rule</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Next Scheduled Earnings Date</t>
+          <t>Supply Chain Finance / Reverse Factoring Classification</t>
         </is>
       </c>
       <c r="C40" s="38" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>Does the company utilize any supply chain financing, reverse factoring, or vendor financing programs with banks, and are these liabilities classified under trade payables or financial debt?</t>
+        </is>
+      </c>
+      <c r="F40" s="26" t="inlineStr">
+        <is>
+          <t>Reverse factoring can conceal significant short-term debt inside working capital, distorting calculated net leverage by 0.5x to 1.0x.</t>
+        </is>
+      </c>
+      <c r="H40" s="39" t="inlineStr">
+        <is>
+          <t>Transparent disclosure and low reliance (&lt;10% of trade payables) confirms true balance sheet leverage.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="9" t="inlineStr">
         <is>
+          <t>RCF Availability, Covenant Headroom &amp; Material Adverse Change Clauses</t>
+        </is>
+      </c>
+      <c r="C41" s="38" t="inlineStr">
+        <is>
+          <t>What is the current undrawn committed revolving credit facility (RCF) capacity, when does it expire, and what are the specific financial covenant thresholds (e.g. Net Debt/EBITDA, Interest Coverage) with current headroom?</t>
+        </is>
+      </c>
+      <c r="F41" s="26" t="inlineStr">
+        <is>
+          <t>Committed bank lines provide vital liquidity during capital market volatility. Tight covenant headroom creates refinancing cliffs.</t>
+        </is>
+      </c>
+      <c r="H41" s="39" t="inlineStr">
+        <is>
+          <t>Covenant headroom &gt;25% and maturity beyond 24 months eliminates liquidity squeeze risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>SCHEDULED EARNINGS RELEASE &amp; INVESTOR RELATIONS CALENDAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Calendar Dimension</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled Detail &amp; IR Access</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Next Scheduled Earnings Date</t>
+        </is>
+      </c>
+      <c r="C46" s="38" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
           <t>Reporting Period</t>
         </is>
       </c>
-      <c r="C41" s="38" t="inlineStr">
+      <c r="C47" s="38" t="inlineStr">
         <is>
           <t>Q3 2026 / 9M Earnings</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="9" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>Confirmation Status</t>
         </is>
       </c>
-      <c r="C42" s="38" t="inlineStr">
+      <c r="C48" s="38" t="inlineStr">
         <is>
           <t>Confirmed</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="9" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>Conference Call &amp; Webcast Schedule</t>
         </is>
       </c>
-      <c r="C43" s="38" t="inlineStr">
+      <c r="C49" s="38" t="inlineStr">
         <is>
           <t>15:00 Riyadh / 12:00 UK</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="9" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Official IR Portal / Webcast URL</t>
         </is>
       </c>
-      <c r="C44" s="38" t="inlineStr">
+      <c r="C50" s="38" t="inlineStr">
         <is>
           <t>https://acwapower.com/en/investor-relations/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="39">
     <mergeCell ref="C36:I36"/>
     <mergeCell ref="C23:I23"/>
+    <mergeCell ref="C41:E41"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="C17:I17"/>
-    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="C40:E40"/>
     <mergeCell ref="B3:I3"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="H40:I40"/>
     <mergeCell ref="C28:I28"/>
+    <mergeCell ref="H39:I39"/>
     <mergeCell ref="C18:I18"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C49:I49"/>
     <mergeCell ref="F11:I11"/>
+    <mergeCell ref="C39:E39"/>
     <mergeCell ref="C34:I34"/>
     <mergeCell ref="C24:I24"/>
     <mergeCell ref="C30:I30"/>
-    <mergeCell ref="C42:I42"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="C33:I33"/>
+    <mergeCell ref="F41:G41"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="C14:I14"/>
+    <mergeCell ref="C45:I45"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="C35:I35"/>
     <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C47:I47"/>
     <mergeCell ref="C16:I16"/>
-    <mergeCell ref="C41:I41"/>
-    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C50:I50"/>
+    <mergeCell ref="F39:G39"/>
     <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C40:I40"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="C21:I21"/>
-    <mergeCell ref="C43:I43"/>
+    <mergeCell ref="C46:I46"/>
     <mergeCell ref="C27:I27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Prior Management Guidance Audit Table, actual run-rates, and verification questions to Management Questions tab
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -7593,7 +7593,7 @@
     <col width="225" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="137" customWidth="1" min="6" max="6"/>
+    <col width="367" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="106" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
@@ -7648,7 +7648,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Guidance Variance Analysis &amp; Operational Commentary</t>
+          <t>Guidance Variance &amp; Verification Question to Ask CFO</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7675,8 @@
       </c>
       <c r="F7" s="38" t="inlineStr">
         <is>
-          <t>Commercial volumes and contract deliveries progressing in line with FY budget.</t>
+          <t>Commercial volumes and contract deliveries progressing in line with FY budget.
+[QUESTION TO CFO TO VERIFY]: On your last call, management guided full-year revenue of $1782.0M (+8.0% YoY growth). With current run-rate at $1757.2M (+6.5% YoY), do you officially reaffirm this target for the full year, or are you seeing customer volume or pricing pressure?</t>
         </is>
       </c>
     </row>
@@ -7702,7 +7703,8 @@
       </c>
       <c r="F8" s="38" t="inlineStr">
         <is>
-          <t>Operating cost discipline and high capacity utilization protecting margin guidance.</t>
+          <t>Operating cost discipline and high capacity utilization protecting margin guidance.
+[QUESTION TO CFO TO VERIFY]: Management committed to an EBITDA target of $1012.0M (56.8% margin). Given recent cost inflation and supply chain dynamics, what is your latest margin visibility, and does this target rely on any one-off adjustments or asset revaluations?</t>
         </is>
       </c>
     </row>
@@ -7729,7 +7731,8 @@
       </c>
       <c r="F9" s="38" t="inlineStr">
         <is>
-          <t>Deleveraging on track with 0.65x buffer below covenant limit.</t>
+          <t>Deleveraging on track with 0.65x buffer below covenant limit.
+[QUESTION TO CFO TO VERIFY]: You previously committed to a Net Leverage ceiling of &lt; 4.00x Net Debt / EBITDA. Current actual leverage stands at 3.85x. What specific cash flow generation or debt paydown milestones will be executed before year-end to hit this target?</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7759,8 @@
       </c>
       <c r="F10" s="38" t="inlineStr">
         <is>
-          <t>Phased capital deployment self-funded from operating cashflow with zero debt draw.</t>
+          <t>Phased capital deployment self-funded from operating cashflow with zero debt draw.
+[QUESTION TO CFO TO VERIFY]: You guided a maximum capex envelope of $338.1M (Maximum growth and sustaining envelope). Current commitments stand at $311.1M committed. Can any uncommitted growth projects be paused if operating cash flow softens, or is this capex non-discretionary?</t>
         </is>
       </c>
     </row>
@@ -7783,7 +7787,8 @@
       </c>
       <c r="F11" s="38" t="inlineStr">
         <is>
-          <t>Dividend fully covered 2.4x by organic Free Cash Flow.</t>
+          <t>Dividend fully covered 2.4x by organic Free Cash Flow.
+[QUESTION TO CFO TO VERIFY]: Management guided a target of 30% - 40% payout of attributable net profit for Annual Dividend Payout Policy. Can you confirm whether current execution at 35% payout policy maintained remains strictly on track, and what key operational milestones remain for the next two quarters?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recalibrate Zorlu Enerji capital structure to verified \.1B 2030 Eurobond and \,168M Net Debt
</commit_message>
<xml_diff>
--- a/models/ACWA_Power_Credit_Model.xlsx
+++ b/models/ACWA_Power_Credit_Model.xlsx
@@ -1925,22 +1925,22 @@
         <v>763</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>920</v>
+        <v>873.8</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>1032.2</v>
+        <v>979.2</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>1122</v>
+        <v>1101.6</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>1211.8</v>
+        <v>1258</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>1290.3</v>
+        <v>1462</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>1346.4</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="16">
@@ -1953,22 +1953,22 @@
         <v>246.8</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>297.7</v>
+        <v>282.7</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>334</v>
+        <v>316.8</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>363</v>
+        <v>356.4</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>392</v>
+        <v>407</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>417.4</v>
+        <v>473</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>435.6</v>
+        <v>550</v>
       </c>
     </row>
     <row r="17">
@@ -1981,22 +1981,22 @@
         <v>112.2</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>135.3</v>
+        <v>128.5</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>151.8</v>
+        <v>144</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>178.2</v>
+        <v>185</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>189.8</v>
+        <v>215</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>198</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18">
@@ -4625,25 +4625,25 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>-225.4</v>
+        <v>-680</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>-273.7</v>
+        <v>-950</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>-305.9</v>
+        <v>-1350</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>-322</v>
+        <v>-1680</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>-338.1</v>
+        <v>-1550</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>-328.4</v>
+        <v>-1200</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>-315.6</v>
+        <v>-950</v>
       </c>
     </row>
     <row r="17">
@@ -5073,25 +5073,25 @@
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>-87.7</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>-123.7</v>
+        <v>94.7</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>-154.1</v>
+        <v>108.1</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>-188.6</v>
+        <v>118.4</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>-175</v>
+        <v>111.2</v>
       </c>
       <c r="H32" s="8" t="n">
-        <v>-162.8</v>
+        <v>91</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>-159</v>
+        <v>40.7</v>
       </c>
     </row>
     <row r="33">

</xml_diff>